<commit_message>
Fix KOGAS config corruption, extraction decimals, and row height
- Fix save_settings corrupting _W keys to 0.0 (e.g. KOGAS_W_COL_JOINT)
- Standardize UI labels for Joint and Loc in KOGAS mode
- Apply clean_v to strip decimal points from extracted Joint, Loc, Welder, Dwg
- Apply row height settings to the first data sheet in RT/KOGAS generation
- Clear repetitive Joint numbers for multi-shot joints in RT/KOGAS for cleaner reports
</commit_message>
<xml_diff>
--- a/Na-aba/home/data/SISGI-KOGAS-RT-001.xlsx
+++ b/Na-aba/home/data/SISGI-KOGAS-RT-001.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jjch2\Desktop\보고서\Project PROVIDENCE\Request\PMI\Na-aba\home\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA4F3DBA-063C-4EBF-9E1C-334DEECF99E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{500826BB-A592-4F9E-BFA2-87180EEC48F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{EBDC5234-EA45-45C7-9BE3-C0C611B2FCE5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EBDC5234-EA45-45C7-9BE3-C0C611B2FCE5}"/>
   </bookViews>
   <sheets>
     <sheet name="RT(갑) 1" sheetId="10" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="232">
   <si>
     <t>□</t>
   </si>
@@ -921,6 +921,42 @@
   </si>
   <si>
     <t>■  Fe                 □  Al</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>KGW-TL-00</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>~</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>용접방법</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>S25C189</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">      시간       4분        30초         35 매</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>x</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Dia.2.5</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Leng.2.5</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>안중~평택(지하차도) 배관이설공사</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
@@ -954,7 +990,7 @@
         <family val="3"/>
         <charset val="129"/>
       </rPr>
-      <t xml:space="preserve">     3     </t>
+      <t xml:space="preserve">     2     </t>
     </r>
     <r>
       <rPr>
@@ -975,96 +1011,6 @@
       </rPr>
       <t>.</t>
     </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>KGW-TL-00</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>~</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>용접방법</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>S25C189</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">      시간       4분        30초         35 매</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>x</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Dia.2.5</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Leng.2.5</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Page  </t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="9"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">   1      </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve"> of </t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="9"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">     3     </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color indexed="9"/>
-        <rFont val="돋움"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>.</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>안중~평택(지하차도) 배관이설공사</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1770,7 +1716,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="356">
+  <cellXfs count="355">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1957,12 +1903,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
@@ -2344,6 +2284,84 @@
     <xf numFmtId="176" fontId="15" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="45" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="44" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="179" fontId="8" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -2518,9 +2536,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2623,6 +2638,39 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="6" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
@@ -2704,39 +2752,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="6" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
@@ -2765,78 +2780,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="45" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="44" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3376,8 +3319,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr bwMode="auto">
         <a:xfrm>
-          <a:off x="1101616" y="7199915"/>
-          <a:ext cx="4791075" cy="969907"/>
+          <a:off x="1099119" y="7109986"/>
+          <a:ext cx="4798235" cy="975622"/>
           <a:chOff x="126" y="703"/>
           <a:chExt cx="571" cy="103"/>
         </a:xfrm>
@@ -8250,8 +8193,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr bwMode="auto">
         <a:xfrm>
-          <a:off x="1280620" y="5997466"/>
-          <a:ext cx="4612071" cy="1126249"/>
+          <a:off x="1289094" y="5912069"/>
+          <a:ext cx="4608260" cy="1121717"/>
           <a:chOff x="150" y="536"/>
           <a:chExt cx="540" cy="120"/>
         </a:xfrm>
@@ -14016,70 +13959,6 @@
       <xdr:spPr bwMode="auto">
         <a:xfrm>
           <a:off x="762000" y="8915400"/>
-          <a:ext cx="2286000" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="line">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="6350">
-          <a:solidFill>
-            <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
-          </a:solidFill>
-          <a:round/>
-          <a:headEnd/>
-          <a:tailEnd/>
-        </a:ln>
-        <a:effectLst/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:noFill/>
-            </a14:hiddenFill>
-          </a:ext>
-          <a:ext uri="{AF507438-7753-43E0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:effectLst>
-                <a:outerShdw dist="35921" dir="2700000" algn="ctr" rotWithShape="0">
-                  <a:srgbClr val="808080"/>
-                </a:outerShdw>
-              </a:effectLst>
-            </a14:hiddenEffects>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>716280</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>144780</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>144780</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="23845" name="Line 166">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EE446D45-8BA6-FF07-4B9E-339D76420E7B}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr>
-          <a:spLocks noChangeShapeType="1"/>
-        </xdr:cNvSpPr>
-      </xdr:nvSpPr>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="762000" y="9227820"/>
           <a:ext cx="2286000" cy="0"/>
         </a:xfrm>
         <a:prstGeom prst="line">
@@ -14652,44 +14531,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="21.75" customHeight="1">
-      <c r="A1" s="249" t="s">
+      <c r="A1" s="199" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="250"/>
-      <c r="C1" s="250"/>
-      <c r="D1" s="250"/>
-      <c r="E1" s="250"/>
-      <c r="F1" s="250"/>
-      <c r="G1" s="250"/>
-      <c r="H1" s="250"/>
-      <c r="I1" s="250"/>
-      <c r="J1" s="250"/>
-      <c r="K1" s="250"/>
-      <c r="L1" s="250"/>
-      <c r="M1" s="250"/>
-      <c r="N1" s="250"/>
-      <c r="O1" s="250"/>
-      <c r="P1" s="250"/>
+      <c r="B1" s="273"/>
+      <c r="C1" s="273"/>
+      <c r="D1" s="273"/>
+      <c r="E1" s="273"/>
+      <c r="F1" s="273"/>
+      <c r="G1" s="273"/>
+      <c r="H1" s="273"/>
+      <c r="I1" s="273"/>
+      <c r="J1" s="273"/>
+      <c r="K1" s="273"/>
+      <c r="L1" s="273"/>
+      <c r="M1" s="273"/>
+      <c r="N1" s="273"/>
+      <c r="O1" s="273"/>
+      <c r="P1" s="273"/>
     </row>
     <row r="2" spans="1:16" ht="18.75" customHeight="1">
-      <c r="A2" s="249" t="s">
+      <c r="A2" s="199" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="250"/>
-      <c r="C2" s="250"/>
-      <c r="D2" s="250"/>
-      <c r="E2" s="250"/>
-      <c r="F2" s="250"/>
-      <c r="G2" s="250"/>
-      <c r="H2" s="250"/>
-      <c r="I2" s="250"/>
-      <c r="J2" s="250"/>
-      <c r="K2" s="250"/>
-      <c r="L2" s="250"/>
-      <c r="M2" s="250"/>
-      <c r="N2" s="250"/>
-      <c r="O2" s="250"/>
-      <c r="P2" s="250"/>
+      <c r="B2" s="273"/>
+      <c r="C2" s="273"/>
+      <c r="D2" s="273"/>
+      <c r="E2" s="273"/>
+      <c r="F2" s="273"/>
+      <c r="G2" s="273"/>
+      <c r="H2" s="273"/>
+      <c r="I2" s="273"/>
+      <c r="J2" s="273"/>
+      <c r="K2" s="273"/>
+      <c r="L2" s="273"/>
+      <c r="M2" s="273"/>
+      <c r="N2" s="273"/>
+      <c r="O2" s="273"/>
+      <c r="P2" s="273"/>
     </row>
     <row r="3" spans="1:16" ht="12" customHeight="1">
       <c r="A3" s="3"/>
@@ -14705,155 +14584,153 @@
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
-      <c r="N3" s="251" t="s">
-        <v>231</v>
-      </c>
-      <c r="O3" s="252"/>
-      <c r="P3" s="252"/>
+      <c r="N3" s="274"/>
+      <c r="O3" s="275"/>
+      <c r="P3" s="275"/>
     </row>
     <row r="4" spans="1:16" ht="15.75" customHeight="1">
       <c r="A4" s="5"/>
       <c r="B4" s="6"/>
-      <c r="C4" s="253" t="s">
+      <c r="C4" s="276" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="254"/>
-      <c r="E4" s="254"/>
-      <c r="F4" s="254"/>
-      <c r="G4" s="254"/>
-      <c r="H4" s="254"/>
-      <c r="I4" s="254"/>
-      <c r="J4" s="254"/>
-      <c r="K4" s="255"/>
-      <c r="L4" s="204" t="s">
+      <c r="D4" s="277"/>
+      <c r="E4" s="277"/>
+      <c r="F4" s="277"/>
+      <c r="G4" s="277"/>
+      <c r="H4" s="277"/>
+      <c r="I4" s="277"/>
+      <c r="J4" s="277"/>
+      <c r="K4" s="278"/>
+      <c r="L4" s="228" t="s">
         <v>4</v>
       </c>
-      <c r="M4" s="205"/>
-      <c r="N4" s="262" t="s">
+      <c r="M4" s="229"/>
+      <c r="N4" s="285" t="s">
         <v>169</v>
       </c>
-      <c r="O4" s="263"/>
-      <c r="P4" s="264"/>
+      <c r="O4" s="286"/>
+      <c r="P4" s="287"/>
     </row>
     <row r="5" spans="1:16" ht="12.75" customHeight="1">
       <c r="A5" s="5"/>
       <c r="B5" s="6"/>
-      <c r="C5" s="256" t="s">
+      <c r="C5" s="279" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="256"/>
-      <c r="E5" s="256"/>
-      <c r="F5" s="256"/>
-      <c r="G5" s="256"/>
-      <c r="H5" s="256"/>
-      <c r="I5" s="256"/>
-      <c r="J5" s="256"/>
-      <c r="K5" s="257"/>
-      <c r="L5" s="206" t="s">
+      <c r="D5" s="279"/>
+      <c r="E5" s="279"/>
+      <c r="F5" s="279"/>
+      <c r="G5" s="279"/>
+      <c r="H5" s="279"/>
+      <c r="I5" s="279"/>
+      <c r="J5" s="279"/>
+      <c r="K5" s="280"/>
+      <c r="L5" s="230" t="s">
         <v>6</v>
       </c>
-      <c r="M5" s="207"/>
-      <c r="N5" s="265"/>
-      <c r="O5" s="266"/>
-      <c r="P5" s="267"/>
+      <c r="M5" s="231"/>
+      <c r="N5" s="288"/>
+      <c r="O5" s="289"/>
+      <c r="P5" s="290"/>
     </row>
     <row r="6" spans="1:16" ht="12.75" customHeight="1">
       <c r="A6" s="5"/>
       <c r="B6" s="6"/>
-      <c r="C6" s="258" t="s">
+      <c r="C6" s="281" t="s">
         <v>168</v>
       </c>
-      <c r="D6" s="258"/>
-      <c r="E6" s="258"/>
-      <c r="F6" s="258"/>
-      <c r="G6" s="258"/>
-      <c r="H6" s="258"/>
-      <c r="I6" s="258"/>
-      <c r="J6" s="258"/>
-      <c r="K6" s="259"/>
-      <c r="L6" s="208" t="s">
+      <c r="D6" s="281"/>
+      <c r="E6" s="281"/>
+      <c r="F6" s="281"/>
+      <c r="G6" s="281"/>
+      <c r="H6" s="281"/>
+      <c r="I6" s="281"/>
+      <c r="J6" s="281"/>
+      <c r="K6" s="282"/>
+      <c r="L6" s="232" t="s">
         <v>7</v>
       </c>
-      <c r="M6" s="209"/>
-      <c r="N6" s="218" t="s">
+      <c r="M6" s="233"/>
+      <c r="N6" s="242" t="s">
         <v>170</v>
       </c>
-      <c r="O6" s="228"/>
-      <c r="P6" s="229"/>
+      <c r="O6" s="252"/>
+      <c r="P6" s="253"/>
     </row>
     <row r="7" spans="1:16" ht="12.75" customHeight="1">
       <c r="A7" s="7"/>
       <c r="B7" s="8"/>
-      <c r="C7" s="260" t="s">
+      <c r="C7" s="283" t="s">
         <v>8</v>
       </c>
-      <c r="D7" s="260"/>
-      <c r="E7" s="260"/>
-      <c r="F7" s="260"/>
-      <c r="G7" s="260"/>
-      <c r="H7" s="260"/>
-      <c r="I7" s="260"/>
-      <c r="J7" s="260"/>
-      <c r="K7" s="261"/>
-      <c r="L7" s="210" t="s">
+      <c r="D7" s="283"/>
+      <c r="E7" s="283"/>
+      <c r="F7" s="283"/>
+      <c r="G7" s="283"/>
+      <c r="H7" s="283"/>
+      <c r="I7" s="283"/>
+      <c r="J7" s="283"/>
+      <c r="K7" s="284"/>
+      <c r="L7" s="234" t="s">
         <v>9</v>
       </c>
-      <c r="M7" s="211"/>
-      <c r="N7" s="230"/>
-      <c r="O7" s="231"/>
-      <c r="P7" s="232"/>
+      <c r="M7" s="235"/>
+      <c r="N7" s="254"/>
+      <c r="O7" s="255"/>
+      <c r="P7" s="256"/>
     </row>
     <row r="8" spans="1:16" s="12" customFormat="1" ht="24" customHeight="1">
       <c r="A8" s="9"/>
       <c r="B8" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="212" t="s">
-        <v>232</v>
-      </c>
-      <c r="D8" s="213"/>
-      <c r="E8" s="213"/>
-      <c r="F8" s="213"/>
-      <c r="G8" s="213"/>
-      <c r="H8" s="213"/>
-      <c r="I8" s="214"/>
+      <c r="C8" s="236" t="s">
+        <v>230</v>
+      </c>
+      <c r="D8" s="237"/>
+      <c r="E8" s="237"/>
+      <c r="F8" s="237"/>
+      <c r="G8" s="237"/>
+      <c r="H8" s="237"/>
+      <c r="I8" s="238"/>
       <c r="J8" s="11"/>
       <c r="K8" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="L8" s="215" t="s">
+      <c r="L8" s="239" t="s">
         <v>206</v>
       </c>
-      <c r="M8" s="216"/>
-      <c r="N8" s="216"/>
-      <c r="O8" s="216"/>
-      <c r="P8" s="217"/>
+      <c r="M8" s="240"/>
+      <c r="N8" s="240"/>
+      <c r="O8" s="240"/>
+      <c r="P8" s="241"/>
     </row>
     <row r="9" spans="1:16" s="12" customFormat="1" ht="13.5" customHeight="1">
       <c r="A9" s="13"/>
       <c r="B9" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="218" t="s">
+      <c r="C9" s="242" t="s">
         <v>205</v>
       </c>
-      <c r="D9" s="219"/>
-      <c r="E9" s="219"/>
-      <c r="F9" s="219"/>
-      <c r="G9" s="219"/>
-      <c r="H9" s="219"/>
-      <c r="I9" s="220"/>
+      <c r="D9" s="243"/>
+      <c r="E9" s="243"/>
+      <c r="F9" s="243"/>
+      <c r="G9" s="243"/>
+      <c r="H9" s="243"/>
+      <c r="I9" s="244"/>
       <c r="J9" s="15"/>
       <c r="K9" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="L9" s="235" t="s">
+      <c r="L9" s="259" t="s">
         <v>217</v>
       </c>
-      <c r="M9" s="236"/>
-      <c r="N9" s="236"/>
-      <c r="O9" s="236"/>
-      <c r="P9" s="118" t="s">
+      <c r="M9" s="260"/>
+      <c r="N9" s="260"/>
+      <c r="O9" s="260"/>
+      <c r="P9" s="116" t="s">
         <v>14</v>
       </c>
     </row>
@@ -14862,22 +14739,22 @@
       <c r="B10" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="221"/>
-      <c r="D10" s="222"/>
-      <c r="E10" s="222"/>
-      <c r="F10" s="222"/>
-      <c r="G10" s="222"/>
-      <c r="H10" s="222"/>
-      <c r="I10" s="223"/>
+      <c r="C10" s="245"/>
+      <c r="D10" s="246"/>
+      <c r="E10" s="246"/>
+      <c r="F10" s="246"/>
+      <c r="G10" s="246"/>
+      <c r="H10" s="246"/>
+      <c r="I10" s="247"/>
       <c r="J10" s="18"/>
       <c r="K10" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="L10" s="237"/>
-      <c r="M10" s="238"/>
-      <c r="N10" s="238"/>
-      <c r="O10" s="238"/>
-      <c r="P10" s="119" t="s">
+      <c r="L10" s="261"/>
+      <c r="M10" s="262"/>
+      <c r="N10" s="262"/>
+      <c r="O10" s="262"/>
+      <c r="P10" s="117" t="s">
         <v>171</v>
       </c>
     </row>
@@ -14886,104 +14763,104 @@
       <c r="B11" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="120" t="s">
+      <c r="C11" s="118" t="s">
         <v>172</v>
       </c>
-      <c r="D11" s="121" t="s">
+      <c r="D11" s="119" t="s">
         <v>19</v>
       </c>
-      <c r="E11" s="121" t="s">
+      <c r="E11" s="119" t="s">
         <v>18</v>
       </c>
-      <c r="F11" s="121" t="s">
+      <c r="F11" s="119" t="s">
         <v>20</v>
       </c>
-      <c r="G11" s="121" t="s">
+      <c r="G11" s="119" t="s">
         <v>18</v>
       </c>
-      <c r="H11" s="121" t="s">
+      <c r="H11" s="119" t="s">
         <v>21</v>
       </c>
-      <c r="I11" s="122"/>
+      <c r="I11" s="120"/>
       <c r="J11" s="15"/>
       <c r="K11" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="L11" s="197" t="s">
+      <c r="L11" s="221" t="s">
         <v>177</v>
       </c>
-      <c r="M11" s="198"/>
-      <c r="N11" s="198"/>
-      <c r="O11" s="198"/>
-      <c r="P11" s="243"/>
+      <c r="M11" s="222"/>
+      <c r="N11" s="222"/>
+      <c r="O11" s="222"/>
+      <c r="P11" s="267"/>
     </row>
     <row r="12" spans="1:16" s="12" customFormat="1" ht="13.5" customHeight="1">
       <c r="A12" s="21"/>
       <c r="B12" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="C12" s="123"/>
-      <c r="D12" s="124" t="s">
+      <c r="C12" s="121"/>
+      <c r="D12" s="122" t="s">
         <v>24</v>
       </c>
-      <c r="E12" s="124"/>
-      <c r="F12" s="124" t="s">
+      <c r="E12" s="122"/>
+      <c r="F12" s="122" t="s">
         <v>25</v>
       </c>
-      <c r="G12" s="124"/>
-      <c r="H12" s="124" t="s">
+      <c r="G12" s="122"/>
+      <c r="H12" s="122" t="s">
         <v>26</v>
       </c>
-      <c r="I12" s="125"/>
+      <c r="I12" s="123"/>
       <c r="J12" s="24"/>
       <c r="K12" s="22" t="s">
-        <v>225</v>
-      </c>
-      <c r="L12" s="244"/>
-      <c r="M12" s="245"/>
-      <c r="N12" s="245"/>
-      <c r="O12" s="245"/>
-      <c r="P12" s="246"/>
+        <v>224</v>
+      </c>
+      <c r="L12" s="268"/>
+      <c r="M12" s="269"/>
+      <c r="N12" s="269"/>
+      <c r="O12" s="269"/>
+      <c r="P12" s="270"/>
     </row>
     <row r="13" spans="1:16" s="12" customFormat="1" ht="13.5" customHeight="1">
       <c r="A13" s="19"/>
       <c r="B13" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="C13" s="120" t="s">
+      <c r="C13" s="118" t="s">
         <v>18</v>
       </c>
-      <c r="D13" s="121" t="s">
+      <c r="D13" s="119" t="s">
         <v>28</v>
       </c>
-      <c r="E13" s="120" t="s">
+      <c r="E13" s="118" t="s">
         <v>18</v>
       </c>
-      <c r="F13" s="121" t="s">
+      <c r="F13" s="119" t="s">
         <v>29</v>
       </c>
-      <c r="G13" s="121" t="s">
+      <c r="G13" s="119" t="s">
         <v>198</v>
       </c>
-      <c r="H13" s="121" t="s">
+      <c r="H13" s="119" t="s">
         <v>30</v>
       </c>
-      <c r="I13" s="122"/>
+      <c r="I13" s="120"/>
       <c r="J13" s="15"/>
       <c r="K13" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="L13" s="139" t="s">
+      <c r="L13" s="137" t="s">
         <v>32</v>
       </c>
-      <c r="M13" s="241">
+      <c r="M13" s="265">
         <v>15.9</v>
       </c>
-      <c r="N13" s="241"/>
-      <c r="O13" s="121" t="s">
+      <c r="N13" s="265"/>
+      <c r="O13" s="119" t="s">
         <v>18</v>
       </c>
-      <c r="P13" s="141" t="s">
+      <c r="P13" s="139" t="s">
         <v>33</v>
       </c>
     </row>
@@ -14992,32 +14869,32 @@
       <c r="B14" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="C14" s="126"/>
-      <c r="D14" s="127" t="s">
+      <c r="C14" s="124"/>
+      <c r="D14" s="125" t="s">
         <v>35</v>
       </c>
-      <c r="E14" s="128"/>
-      <c r="F14" s="127" t="s">
+      <c r="E14" s="126"/>
+      <c r="F14" s="125" t="s">
         <v>36</v>
       </c>
-      <c r="G14" s="127"/>
-      <c r="H14" s="127" t="s">
+      <c r="G14" s="125"/>
+      <c r="H14" s="125" t="s">
         <v>37</v>
       </c>
-      <c r="I14" s="129"/>
+      <c r="I14" s="127"/>
       <c r="J14" s="18"/>
       <c r="K14" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="L14" s="142" t="s">
+      <c r="L14" s="140" t="s">
         <v>39</v>
       </c>
-      <c r="M14" s="242"/>
-      <c r="N14" s="242"/>
-      <c r="O14" s="124" t="s">
+      <c r="M14" s="266"/>
+      <c r="N14" s="266"/>
+      <c r="O14" s="122" t="s">
         <v>173</v>
       </c>
-      <c r="P14" s="144" t="s">
+      <c r="P14" s="142" t="s">
         <v>40</v>
       </c>
     </row>
@@ -15026,36 +14903,36 @@
       <c r="B15" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="C15" s="120" t="s">
+      <c r="C15" s="118" t="s">
         <v>172</v>
       </c>
-      <c r="D15" s="233" t="s">
+      <c r="D15" s="257" t="s">
         <v>42</v>
       </c>
-      <c r="E15" s="234"/>
-      <c r="F15" s="234"/>
-      <c r="G15" s="121" t="s">
+      <c r="E15" s="258"/>
+      <c r="F15" s="258"/>
+      <c r="G15" s="119" t="s">
         <v>164</v>
       </c>
-      <c r="H15" s="233" t="s">
+      <c r="H15" s="257" t="s">
         <v>43</v>
       </c>
-      <c r="I15" s="295"/>
+      <c r="I15" s="329"/>
       <c r="J15" s="15"/>
       <c r="K15" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="L15" s="145" t="s">
+      <c r="L15" s="143" t="s">
         <v>207</v>
       </c>
-      <c r="M15" s="239">
+      <c r="M15" s="263">
         <v>2</v>
       </c>
-      <c r="N15" s="239"/>
-      <c r="O15" s="121" t="s">
+      <c r="N15" s="263"/>
+      <c r="O15" s="119" t="s">
         <v>18</v>
       </c>
-      <c r="P15" s="141" t="s">
+      <c r="P15" s="139" t="s">
         <v>33</v>
       </c>
     </row>
@@ -15064,34 +14941,34 @@
       <c r="B16" s="22" t="s">
         <v>45</v>
       </c>
-      <c r="C16" s="123" t="s">
+      <c r="C16" s="121" t="s">
         <v>172</v>
       </c>
-      <c r="D16" s="247" t="s">
+      <c r="D16" s="271" t="s">
         <v>46</v>
       </c>
-      <c r="E16" s="248"/>
-      <c r="F16" s="248"/>
-      <c r="G16" s="124" t="s">
+      <c r="E16" s="272"/>
+      <c r="F16" s="272"/>
+      <c r="G16" s="122" t="s">
         <v>18</v>
       </c>
-      <c r="H16" s="247" t="s">
+      <c r="H16" s="271" t="s">
         <v>47</v>
       </c>
-      <c r="I16" s="275"/>
+      <c r="I16" s="298"/>
       <c r="J16" s="24"/>
       <c r="K16" s="22" t="s">
         <v>48</v>
       </c>
-      <c r="L16" s="133" t="s">
+      <c r="L16" s="131" t="s">
         <v>49</v>
       </c>
-      <c r="M16" s="240"/>
-      <c r="N16" s="240"/>
-      <c r="O16" s="124" t="s">
+      <c r="M16" s="264"/>
+      <c r="N16" s="264"/>
+      <c r="O16" s="122" t="s">
         <v>173</v>
       </c>
-      <c r="P16" s="140" t="s">
+      <c r="P16" s="138" t="s">
         <v>40</v>
       </c>
     </row>
@@ -15100,81 +14977,81 @@
       <c r="B17" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="C17" s="120" t="s">
+      <c r="C17" s="118" t="s">
         <v>18</v>
       </c>
-      <c r="D17" s="130" t="s">
+      <c r="D17" s="128" t="s">
         <v>51</v>
       </c>
-      <c r="E17" s="131"/>
-      <c r="F17" s="130"/>
-      <c r="G17" s="121" t="s">
+      <c r="E17" s="129"/>
+      <c r="F17" s="128"/>
+      <c r="G17" s="119" t="s">
         <v>173</v>
       </c>
-      <c r="H17" s="130" t="s">
+      <c r="H17" s="128" t="s">
         <v>174</v>
       </c>
-      <c r="I17" s="132"/>
+      <c r="I17" s="130"/>
       <c r="J17" s="15"/>
       <c r="K17" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="L17" s="298" t="s">
+      <c r="L17" s="332" t="s">
         <v>178</v>
       </c>
-      <c r="M17" s="299"/>
-      <c r="N17" s="299"/>
-      <c r="O17" s="299"/>
-      <c r="P17" s="300"/>
+      <c r="M17" s="333"/>
+      <c r="N17" s="333"/>
+      <c r="O17" s="333"/>
+      <c r="P17" s="334"/>
     </row>
     <row r="18" spans="1:16" s="12" customFormat="1" ht="12.75" customHeight="1">
       <c r="A18" s="13"/>
       <c r="B18" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="C18" s="133"/>
-      <c r="D18" s="134">
+      <c r="C18" s="131"/>
+      <c r="D18" s="132">
         <v>55</v>
       </c>
-      <c r="E18" s="135" t="s">
+      <c r="E18" s="133" t="s">
         <v>175</v>
       </c>
-      <c r="F18" s="136" t="s">
+      <c r="F18" s="134" t="s">
         <v>176</v>
       </c>
-      <c r="G18" s="137"/>
-      <c r="H18" s="134" t="s">
-        <v>226</v>
-      </c>
-      <c r="I18" s="138"/>
+      <c r="G18" s="135"/>
+      <c r="H18" s="132" t="s">
+        <v>225</v>
+      </c>
+      <c r="I18" s="136"/>
       <c r="J18" s="18"/>
       <c r="K18" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="L18" s="301" t="s">
+      <c r="L18" s="335" t="s">
         <v>179</v>
       </c>
-      <c r="M18" s="302"/>
-      <c r="N18" s="302"/>
-      <c r="O18" s="302"/>
-      <c r="P18" s="303"/>
+      <c r="M18" s="336"/>
+      <c r="N18" s="336"/>
+      <c r="O18" s="336"/>
+      <c r="P18" s="337"/>
     </row>
     <row r="19" spans="1:16" s="31" customFormat="1" ht="13.5" customHeight="1">
       <c r="A19" s="28"/>
       <c r="B19" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="C19" s="293" t="s">
+      <c r="C19" s="327" t="s">
         <v>56</v>
       </c>
-      <c r="D19" s="326" t="s">
+      <c r="D19" s="349" t="s">
+        <v>228</v>
+      </c>
+      <c r="E19" s="351" t="s">
+        <v>227</v>
+      </c>
+      <c r="F19" s="347" t="s">
         <v>229</v>
-      </c>
-      <c r="E19" s="328" t="s">
-        <v>228</v>
-      </c>
-      <c r="F19" s="324" t="s">
-        <v>230</v>
       </c>
       <c r="G19" s="20" t="s">
         <v>18</v>
@@ -15187,15 +15064,15 @@
       <c r="K19" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="L19" s="117"/>
-      <c r="M19" s="131" t="s">
+      <c r="L19" s="115"/>
+      <c r="M19" s="129" t="s">
         <v>180</v>
       </c>
-      <c r="N19" s="131"/>
-      <c r="O19" s="121" t="s">
+      <c r="N19" s="129"/>
+      <c r="O19" s="119" t="s">
         <v>18</v>
       </c>
-      <c r="P19" s="141" t="s">
+      <c r="P19" s="139" t="s">
         <v>33</v>
       </c>
     </row>
@@ -15204,10 +15081,10 @@
       <c r="B20" s="22" t="s">
         <v>60</v>
       </c>
-      <c r="C20" s="294"/>
-      <c r="D20" s="327"/>
-      <c r="E20" s="329"/>
-      <c r="F20" s="325"/>
+      <c r="C20" s="328"/>
+      <c r="D20" s="350"/>
+      <c r="E20" s="352"/>
+      <c r="F20" s="348"/>
       <c r="G20" s="23" t="s">
         <v>173</v>
       </c>
@@ -15219,47 +15096,47 @@
       <c r="K20" s="22" t="s">
         <v>62</v>
       </c>
-      <c r="L20" s="306" t="s">
+      <c r="L20" s="340" t="s">
         <v>181</v>
       </c>
-      <c r="M20" s="242"/>
-      <c r="N20" s="242"/>
-      <c r="O20" s="124" t="s">
+      <c r="M20" s="266"/>
+      <c r="N20" s="266"/>
+      <c r="O20" s="122" t="s">
         <v>164</v>
       </c>
-      <c r="P20" s="140" t="s">
+      <c r="P20" s="138" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="21" spans="1:16" s="31" customFormat="1" ht="13.5" customHeight="1">
       <c r="A21" s="28"/>
-      <c r="B21" s="116" t="s">
+      <c r="B21" s="114" t="s">
         <v>166</v>
       </c>
-      <c r="C21" s="280" t="s">
+      <c r="C21" s="303" t="s">
         <v>167</v>
       </c>
-      <c r="D21" s="281"/>
-      <c r="E21" s="281"/>
-      <c r="F21" s="281"/>
-      <c r="G21" s="281"/>
-      <c r="H21" s="281"/>
-      <c r="I21" s="296"/>
+      <c r="D21" s="304"/>
+      <c r="E21" s="304"/>
+      <c r="F21" s="304"/>
+      <c r="G21" s="304"/>
+      <c r="H21" s="304"/>
+      <c r="I21" s="330"/>
       <c r="J21" s="30"/>
       <c r="K21" s="14" t="s">
         <v>213</v>
       </c>
-      <c r="L21" s="179"/>
-      <c r="M21" s="180" t="s">
+      <c r="L21" s="177"/>
+      <c r="M21" s="178" t="s">
         <v>173</v>
       </c>
-      <c r="N21" s="180" t="s">
+      <c r="N21" s="178" t="s">
         <v>215</v>
       </c>
-      <c r="O21" s="180" t="s">
+      <c r="O21" s="178" t="s">
         <v>164</v>
       </c>
-      <c r="P21" s="183" t="s">
+      <c r="P21" s="181" t="s">
         <v>216</v>
       </c>
     </row>
@@ -15268,328 +15145,328 @@
       <c r="B22" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="C22" s="282" t="s">
-        <v>227</v>
-      </c>
-      <c r="D22" s="283"/>
-      <c r="E22" s="283"/>
-      <c r="F22" s="283"/>
-      <c r="G22" s="283"/>
-      <c r="H22" s="283"/>
-      <c r="I22" s="297"/>
+      <c r="C22" s="305" t="s">
+        <v>226</v>
+      </c>
+      <c r="D22" s="306"/>
+      <c r="E22" s="306"/>
+      <c r="F22" s="306"/>
+      <c r="G22" s="306"/>
+      <c r="H22" s="306"/>
+      <c r="I22" s="331"/>
       <c r="J22" s="34"/>
       <c r="K22" s="22" t="s">
         <v>214</v>
       </c>
-      <c r="L22" s="181"/>
-      <c r="M22" s="176" t="s">
+      <c r="L22" s="179"/>
+      <c r="M22" s="174" t="s">
         <v>164</v>
       </c>
-      <c r="N22" s="176" t="s">
+      <c r="N22" s="174" t="s">
         <v>218</v>
       </c>
-      <c r="O22" s="176" t="s">
+      <c r="O22" s="174" t="s">
         <v>164</v>
       </c>
-      <c r="P22" s="184" t="s">
+      <c r="P22" s="182" t="s">
         <v>219</v>
       </c>
     </row>
     <row r="23" spans="1:16" s="31" customFormat="1" ht="23.1" customHeight="1">
-      <c r="A23" s="115"/>
-      <c r="B23" s="127" t="s">
+      <c r="A23" s="113"/>
+      <c r="B23" s="125" t="s">
         <v>186</v>
       </c>
-      <c r="C23" s="126"/>
-      <c r="D23" s="147" t="s">
+      <c r="C23" s="124"/>
+      <c r="D23" s="145" t="s">
         <v>187</v>
       </c>
-      <c r="E23" s="330">
+      <c r="E23" s="353">
         <v>375</v>
       </c>
-      <c r="F23" s="331"/>
-      <c r="G23" s="121" t="s">
+      <c r="F23" s="354"/>
+      <c r="G23" s="119" t="s">
         <v>18</v>
       </c>
-      <c r="H23" s="121" t="s">
+      <c r="H23" s="119" t="s">
         <v>58</v>
       </c>
-      <c r="I23" s="148"/>
+      <c r="I23" s="146"/>
       <c r="J23" s="37"/>
       <c r="K23" s="14" t="s">
         <v>203</v>
       </c>
-      <c r="L23" s="315" t="s">
+      <c r="L23" s="311" t="s">
         <v>210</v>
       </c>
-      <c r="M23" s="316"/>
-      <c r="N23" s="316"/>
-      <c r="O23" s="313" t="s">
+      <c r="M23" s="312"/>
+      <c r="N23" s="312"/>
+      <c r="O23" s="309" t="s">
         <v>211</v>
       </c>
-      <c r="P23" s="314"/>
+      <c r="P23" s="310"/>
     </row>
     <row r="24" spans="1:16" s="31" customFormat="1" ht="23.1" customHeight="1">
-      <c r="A24" s="115"/>
-      <c r="B24" s="127" t="s">
+      <c r="A24" s="113"/>
+      <c r="B24" s="125" t="s">
         <v>188</v>
       </c>
-      <c r="C24" s="126"/>
-      <c r="D24" s="147" t="s">
+      <c r="C24" s="124"/>
+      <c r="D24" s="145" t="s">
         <v>189</v>
       </c>
-      <c r="E24" s="276">
+      <c r="E24" s="299">
         <v>17.899999999999999</v>
       </c>
-      <c r="F24" s="277"/>
-      <c r="G24" s="127" t="s">
+      <c r="F24" s="300"/>
+      <c r="G24" s="125" t="s">
         <v>173</v>
       </c>
-      <c r="H24" s="127" t="s">
+      <c r="H24" s="125" t="s">
         <v>61</v>
       </c>
-      <c r="I24" s="148"/>
+      <c r="I24" s="146"/>
       <c r="J24" s="40"/>
-      <c r="K24" s="178" t="s">
+      <c r="K24" s="176" t="s">
         <v>204</v>
       </c>
-      <c r="L24" s="315" t="s">
+      <c r="L24" s="311" t="s">
         <v>220</v>
       </c>
-      <c r="M24" s="316"/>
-      <c r="N24" s="316"/>
-      <c r="O24" s="311" t="s">
+      <c r="M24" s="312"/>
+      <c r="N24" s="312"/>
+      <c r="O24" s="307" t="s">
         <v>221</v>
       </c>
-      <c r="P24" s="312"/>
+      <c r="P24" s="308"/>
     </row>
     <row r="25" spans="1:16" s="31" customFormat="1" ht="13.5" customHeight="1">
       <c r="A25" s="28"/>
-      <c r="B25" s="121" t="s">
+      <c r="B25" s="119" t="s">
         <v>64</v>
       </c>
-      <c r="C25" s="120"/>
-      <c r="D25" s="322" t="s">
+      <c r="C25" s="118"/>
+      <c r="D25" s="345" t="s">
         <v>209</v>
       </c>
-      <c r="E25" s="323"/>
-      <c r="F25" s="323"/>
-      <c r="G25" s="121" t="s">
+      <c r="E25" s="346"/>
+      <c r="F25" s="346"/>
+      <c r="G25" s="119" t="s">
         <v>173</v>
       </c>
-      <c r="H25" s="121" t="s">
+      <c r="H25" s="119" t="s">
         <v>58</v>
       </c>
-      <c r="I25" s="149"/>
+      <c r="I25" s="147"/>
       <c r="J25" s="30"/>
       <c r="K25" s="14" t="s">
         <v>65</v>
       </c>
-      <c r="L25" s="145" t="s">
+      <c r="L25" s="143" t="s">
         <v>66</v>
       </c>
-      <c r="M25" s="239" t="s">
+      <c r="M25" s="263" t="s">
         <v>182</v>
       </c>
-      <c r="N25" s="239"/>
-      <c r="O25" s="239"/>
-      <c r="P25" s="307"/>
+      <c r="N25" s="263"/>
+      <c r="O25" s="263"/>
+      <c r="P25" s="341"/>
     </row>
     <row r="26" spans="1:16" s="31" customFormat="1" ht="13.5" customHeight="1">
       <c r="A26" s="35"/>
-      <c r="B26" s="150" t="s">
+      <c r="B26" s="148" t="s">
         <v>67</v>
       </c>
-      <c r="C26" s="126"/>
-      <c r="D26" s="151" t="s">
+      <c r="C26" s="124"/>
+      <c r="D26" s="149" t="s">
         <v>190</v>
       </c>
-      <c r="E26" s="128" t="s">
+      <c r="E26" s="126" t="s">
         <v>57</v>
       </c>
-      <c r="F26" s="152">
+      <c r="F26" s="150">
         <v>17</v>
       </c>
-      <c r="G26" s="127" t="s">
+      <c r="G26" s="125" t="s">
         <v>18</v>
       </c>
-      <c r="H26" s="127" t="s">
+      <c r="H26" s="125" t="s">
         <v>61</v>
       </c>
-      <c r="I26" s="148"/>
+      <c r="I26" s="146"/>
       <c r="J26" s="37"/>
       <c r="K26" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="L26" s="126" t="s">
+      <c r="L26" s="124" t="s">
         <v>69</v>
       </c>
-      <c r="M26" s="240" t="s">
+      <c r="M26" s="264" t="s">
         <v>183</v>
       </c>
-      <c r="N26" s="240"/>
-      <c r="O26" s="240"/>
-      <c r="P26" s="308"/>
+      <c r="N26" s="264"/>
+      <c r="O26" s="264"/>
+      <c r="P26" s="342"/>
     </row>
     <row r="27" spans="1:16" s="31" customFormat="1" ht="13.5" customHeight="1">
       <c r="A27" s="28"/>
-      <c r="B27" s="153" t="s">
+      <c r="B27" s="151" t="s">
         <v>70</v>
       </c>
-      <c r="C27" s="298"/>
-      <c r="D27" s="309" t="s">
+      <c r="C27" s="332"/>
+      <c r="D27" s="343" t="s">
         <v>191</v>
       </c>
-      <c r="E27" s="299"/>
-      <c r="F27" s="299" t="s">
+      <c r="E27" s="333"/>
+      <c r="F27" s="333" t="s">
         <v>192</v>
       </c>
-      <c r="G27" s="121" t="s">
+      <c r="G27" s="119" t="s">
         <v>173</v>
       </c>
-      <c r="H27" s="121" t="s">
+      <c r="H27" s="119" t="s">
         <v>71</v>
       </c>
-      <c r="I27" s="149"/>
+      <c r="I27" s="147"/>
       <c r="J27" s="30"/>
       <c r="K27" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="L27" s="117">
+      <c r="L27" s="115">
         <v>1</v>
       </c>
-      <c r="M27" s="121" t="s">
+      <c r="M27" s="119" t="s">
         <v>172</v>
       </c>
-      <c r="N27" s="121" t="s">
+      <c r="N27" s="119" t="s">
         <v>73</v>
       </c>
-      <c r="O27" s="121" t="s">
+      <c r="O27" s="119" t="s">
         <v>18</v>
       </c>
-      <c r="P27" s="141" t="s">
+      <c r="P27" s="139" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="28" spans="1:16" s="31" customFormat="1" ht="13.5" customHeight="1">
       <c r="A28" s="32"/>
-      <c r="B28" s="154" t="s">
+      <c r="B28" s="152" t="s">
         <v>75</v>
       </c>
-      <c r="C28" s="301"/>
-      <c r="D28" s="310"/>
-      <c r="E28" s="302"/>
-      <c r="F28" s="302"/>
-      <c r="G28" s="124" t="s">
+      <c r="C28" s="335"/>
+      <c r="D28" s="344"/>
+      <c r="E28" s="336"/>
+      <c r="F28" s="336"/>
+      <c r="G28" s="122" t="s">
         <v>18</v>
       </c>
-      <c r="H28" s="124" t="s">
+      <c r="H28" s="122" t="s">
         <v>76</v>
       </c>
-      <c r="I28" s="155"/>
+      <c r="I28" s="153"/>
       <c r="J28" s="34"/>
       <c r="K28" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="L28" s="146"/>
-      <c r="M28" s="124" t="s">
+      <c r="L28" s="144"/>
+      <c r="M28" s="122" t="s">
         <v>18</v>
       </c>
-      <c r="N28" s="124" t="s">
+      <c r="N28" s="122" t="s">
         <v>78</v>
       </c>
-      <c r="O28" s="143"/>
-      <c r="P28" s="140"/>
+      <c r="O28" s="141"/>
+      <c r="P28" s="138"/>
     </row>
     <row r="29" spans="1:16" s="31" customFormat="1" ht="23.25" customHeight="1">
       <c r="A29" s="39"/>
-      <c r="B29" s="156" t="s">
+      <c r="B29" s="154" t="s">
         <v>79</v>
       </c>
-      <c r="C29" s="317" t="s">
+      <c r="C29" s="313" t="s">
         <v>193</v>
       </c>
-      <c r="D29" s="318"/>
-      <c r="E29" s="319"/>
-      <c r="F29" s="319"/>
-      <c r="G29" s="319"/>
-      <c r="H29" s="320"/>
-      <c r="I29" s="321"/>
+      <c r="D29" s="314"/>
+      <c r="E29" s="315"/>
+      <c r="F29" s="315"/>
+      <c r="G29" s="315"/>
+      <c r="H29" s="316"/>
+      <c r="I29" s="317"/>
       <c r="J29" s="40"/>
       <c r="K29" s="41" t="s">
         <v>80</v>
       </c>
-      <c r="L29" s="199">
+      <c r="L29" s="223">
         <v>0.32</v>
       </c>
-      <c r="M29" s="200"/>
-      <c r="N29" s="200"/>
-      <c r="O29" s="200"/>
-      <c r="P29" s="201"/>
+      <c r="M29" s="224"/>
+      <c r="N29" s="224"/>
+      <c r="O29" s="224"/>
+      <c r="P29" s="225"/>
     </row>
     <row r="30" spans="1:16" s="31" customFormat="1" ht="12.75" customHeight="1">
       <c r="A30" s="28"/>
-      <c r="B30" s="121" t="s">
+      <c r="B30" s="119" t="s">
         <v>81</v>
       </c>
-      <c r="C30" s="224" t="s">
+      <c r="C30" s="248" t="s">
         <v>200</v>
       </c>
-      <c r="D30" s="225"/>
-      <c r="E30" s="225"/>
-      <c r="F30" s="225"/>
-      <c r="G30" s="121" t="s">
+      <c r="D30" s="249"/>
+      <c r="E30" s="249"/>
+      <c r="F30" s="249"/>
+      <c r="G30" s="119" t="s">
         <v>164</v>
       </c>
-      <c r="H30" s="157" t="s">
+      <c r="H30" s="155" t="s">
         <v>82</v>
       </c>
-      <c r="I30" s="149"/>
+      <c r="I30" s="147"/>
       <c r="J30" s="30"/>
       <c r="K30" s="14" t="s">
         <v>83</v>
       </c>
-      <c r="L30" s="197" t="s">
+      <c r="L30" s="221" t="s">
         <v>202</v>
       </c>
-      <c r="M30" s="198"/>
-      <c r="N30" s="198"/>
-      <c r="O30" s="198"/>
-      <c r="P30" s="177" t="s">
+      <c r="M30" s="222"/>
+      <c r="N30" s="222"/>
+      <c r="O30" s="222"/>
+      <c r="P30" s="175" t="s">
         <v>184</v>
       </c>
     </row>
     <row r="31" spans="1:16" s="31" customFormat="1" ht="12.75" customHeight="1">
       <c r="A31" s="42"/>
-      <c r="B31" s="158" t="s">
+      <c r="B31" s="156" t="s">
         <v>84</v>
       </c>
-      <c r="C31" s="226"/>
-      <c r="D31" s="227"/>
-      <c r="E31" s="227"/>
-      <c r="F31" s="227"/>
+      <c r="C31" s="250"/>
+      <c r="D31" s="251"/>
+      <c r="E31" s="251"/>
+      <c r="F31" s="251"/>
       <c r="G31" s="43" t="s">
         <v>194</v>
       </c>
-      <c r="H31" s="159" t="s">
+      <c r="H31" s="157" t="s">
         <v>85</v>
       </c>
-      <c r="I31" s="160"/>
+      <c r="I31" s="158"/>
       <c r="J31" s="44"/>
       <c r="K31" s="43" t="s">
         <v>86</v>
       </c>
-      <c r="L31" s="194" t="s">
+      <c r="L31" s="218" t="s">
         <v>185</v>
       </c>
-      <c r="M31" s="195"/>
-      <c r="N31" s="195"/>
-      <c r="O31" s="195"/>
-      <c r="P31" s="196"/>
+      <c r="M31" s="219"/>
+      <c r="N31" s="219"/>
+      <c r="O31" s="219"/>
+      <c r="P31" s="220"/>
     </row>
     <row r="32" spans="1:16" s="31" customFormat="1" ht="6.75" customHeight="1">
       <c r="A32" s="35"/>
-      <c r="B32" s="202" t="s">
+      <c r="B32" s="226" t="s">
         <v>87</v>
       </c>
       <c r="C32" s="45"/>
@@ -15609,7 +15486,7 @@
     </row>
     <row r="33" spans="1:16" s="31" customFormat="1" ht="13.5" customHeight="1">
       <c r="A33" s="35"/>
-      <c r="B33" s="203"/>
+      <c r="B33" s="227"/>
       <c r="C33" s="25" t="s">
         <v>165</v>
       </c>
@@ -15804,118 +15681,118 @@
       <c r="B43" s="51" t="s">
         <v>88</v>
       </c>
-      <c r="C43" s="289"/>
-      <c r="D43" s="289"/>
-      <c r="E43" s="289"/>
-      <c r="F43" s="304" t="s">
+      <c r="C43" s="323"/>
+      <c r="D43" s="323"/>
+      <c r="E43" s="323"/>
+      <c r="F43" s="338" t="s">
         <v>89</v>
       </c>
-      <c r="G43" s="305"/>
-      <c r="H43" s="161"/>
+      <c r="G43" s="339"/>
+      <c r="H43" s="159"/>
       <c r="I43" s="52"/>
       <c r="J43" s="53"/>
-      <c r="K43" s="290" t="s">
+      <c r="K43" s="324" t="s">
         <v>197</v>
       </c>
-      <c r="L43" s="291"/>
-      <c r="M43" s="291"/>
-      <c r="N43" s="291"/>
-      <c r="O43" s="291"/>
-      <c r="P43" s="292"/>
+      <c r="L43" s="325"/>
+      <c r="M43" s="325"/>
+      <c r="N43" s="325"/>
+      <c r="O43" s="325"/>
+      <c r="P43" s="326"/>
     </row>
     <row r="44" spans="1:16" ht="15.75" customHeight="1">
       <c r="A44" s="55"/>
       <c r="B44" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="C44" s="271" t="s">
+      <c r="C44" s="294" t="s">
         <v>195</v>
       </c>
-      <c r="D44" s="271"/>
-      <c r="E44" s="271"/>
-      <c r="F44" s="278" t="s">
+      <c r="D44" s="294"/>
+      <c r="E44" s="294"/>
+      <c r="F44" s="301" t="s">
         <v>91</v>
       </c>
-      <c r="G44" s="279"/>
-      <c r="H44" s="128" t="s">
+      <c r="G44" s="302"/>
+      <c r="H44" s="126" t="s">
         <v>196</v>
       </c>
-      <c r="K44" s="191">
+      <c r="K44" s="215">
         <v>45821</v>
       </c>
-      <c r="L44" s="191"/>
-      <c r="M44" s="182" t="s">
-        <v>224</v>
-      </c>
-      <c r="N44" s="192">
+      <c r="L44" s="215"/>
+      <c r="M44" s="180" t="s">
+        <v>223</v>
+      </c>
+      <c r="N44" s="216">
         <v>45827</v>
       </c>
-      <c r="O44" s="192"/>
-      <c r="P44" s="193"/>
+      <c r="O44" s="216"/>
+      <c r="P44" s="217"/>
     </row>
     <row r="45" spans="1:16" ht="12.75" customHeight="1">
       <c r="A45" s="55"/>
       <c r="B45" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C45" s="271"/>
-      <c r="D45" s="271"/>
-      <c r="E45" s="271"/>
-      <c r="F45" s="278" t="s">
+      <c r="C45" s="294"/>
+      <c r="D45" s="294"/>
+      <c r="E45" s="294"/>
+      <c r="F45" s="301" t="s">
         <v>89</v>
       </c>
-      <c r="G45" s="279"/>
-      <c r="H45" s="128"/>
+      <c r="G45" s="302"/>
+      <c r="H45" s="126"/>
       <c r="I45" s="49"/>
       <c r="J45" s="15"/>
-      <c r="K45" s="268" t="s">
+      <c r="K45" s="291" t="s">
         <v>93</v>
       </c>
-      <c r="L45" s="269"/>
-      <c r="M45" s="269"/>
-      <c r="N45" s="269"/>
-      <c r="O45" s="269"/>
-      <c r="P45" s="270"/>
+      <c r="L45" s="292"/>
+      <c r="M45" s="292"/>
+      <c r="N45" s="292"/>
+      <c r="O45" s="292"/>
+      <c r="P45" s="293"/>
     </row>
     <row r="46" spans="1:16" ht="15" customHeight="1">
       <c r="A46" s="55"/>
       <c r="B46" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="C46" s="271" t="s">
+      <c r="C46" s="294" t="s">
         <v>208</v>
       </c>
-      <c r="D46" s="271"/>
-      <c r="E46" s="271"/>
-      <c r="F46" s="278" t="s">
+      <c r="D46" s="294"/>
+      <c r="E46" s="294"/>
+      <c r="F46" s="301" t="s">
         <v>91</v>
       </c>
-      <c r="G46" s="279"/>
-      <c r="H46" s="128" t="s">
+      <c r="G46" s="302"/>
+      <c r="H46" s="126" t="s">
         <v>212</v>
       </c>
       <c r="I46" s="49"/>
       <c r="J46" s="24"/>
-      <c r="K46" s="272"/>
-      <c r="L46" s="273"/>
-      <c r="M46" s="273"/>
-      <c r="N46" s="273"/>
-      <c r="O46" s="273"/>
-      <c r="P46" s="274"/>
+      <c r="K46" s="295"/>
+      <c r="L46" s="296"/>
+      <c r="M46" s="296"/>
+      <c r="N46" s="296"/>
+      <c r="O46" s="296"/>
+      <c r="P46" s="297"/>
     </row>
     <row r="47" spans="1:16" ht="13.5" customHeight="1">
       <c r="A47" s="55"/>
       <c r="B47" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="C47" s="271"/>
-      <c r="D47" s="271"/>
-      <c r="E47" s="271"/>
-      <c r="F47" s="278" t="s">
+      <c r="C47" s="294"/>
+      <c r="D47" s="294"/>
+      <c r="E47" s="294"/>
+      <c r="F47" s="301" t="s">
         <v>89</v>
       </c>
-      <c r="G47" s="279"/>
-      <c r="H47" s="128"/>
+      <c r="G47" s="302"/>
+      <c r="H47" s="126"/>
       <c r="K47" s="38" t="s">
         <v>96</v>
       </c>
@@ -15936,26 +15813,26 @@
       <c r="B48" s="57" t="s">
         <v>99</v>
       </c>
-      <c r="C48" s="288" t="s">
+      <c r="C48" s="322" t="s">
         <v>208</v>
       </c>
-      <c r="D48" s="288"/>
-      <c r="E48" s="288"/>
-      <c r="F48" s="287" t="s">
+      <c r="D48" s="322"/>
+      <c r="E48" s="322"/>
+      <c r="F48" s="321" t="s">
         <v>91</v>
       </c>
-      <c r="G48" s="252"/>
-      <c r="H48" s="162" t="s">
+      <c r="G48" s="275"/>
+      <c r="H48" s="160" t="s">
         <v>212</v>
       </c>
       <c r="I48" s="58"/>
       <c r="J48" s="59"/>
-      <c r="K48" s="284"/>
-      <c r="L48" s="285"/>
-      <c r="M48" s="285"/>
-      <c r="N48" s="285"/>
-      <c r="O48" s="285"/>
-      <c r="P48" s="286"/>
+      <c r="K48" s="318"/>
+      <c r="L48" s="319"/>
+      <c r="M48" s="319"/>
+      <c r="N48" s="319"/>
+      <c r="O48" s="319"/>
+      <c r="P48" s="320"/>
     </row>
   </sheetData>
   <mergeCells count="74">
@@ -16062,1017 +15939,1013 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="39" customHeight="1">
-      <c r="A1" s="249" t="s">
+      <c r="A1" s="199" t="s">
         <v>100</v>
       </c>
-      <c r="B1" s="249"/>
-      <c r="C1" s="249"/>
-      <c r="D1" s="249"/>
-      <c r="E1" s="249"/>
-      <c r="F1" s="249"/>
-      <c r="G1" s="249"/>
-      <c r="H1" s="249"/>
-      <c r="I1" s="249"/>
-      <c r="J1" s="249"/>
-      <c r="K1" s="249"/>
-      <c r="L1" s="249"/>
-      <c r="M1" s="249"/>
-      <c r="N1" s="249"/>
-      <c r="O1" s="249"/>
-      <c r="P1" s="249"/>
-      <c r="Q1" s="249"/>
-      <c r="R1" s="249"/>
-      <c r="S1" s="249"/>
-      <c r="T1" s="249"/>
-      <c r="U1" s="249"/>
-      <c r="V1" s="249"/>
-      <c r="W1" s="249"/>
-      <c r="X1" s="249"/>
+      <c r="B1" s="199"/>
+      <c r="C1" s="199"/>
+      <c r="D1" s="199"/>
+      <c r="E1" s="199"/>
+      <c r="F1" s="199"/>
+      <c r="G1" s="199"/>
+      <c r="H1" s="199"/>
+      <c r="I1" s="199"/>
+      <c r="J1" s="199"/>
+      <c r="K1" s="199"/>
+      <c r="L1" s="199"/>
+      <c r="M1" s="199"/>
+      <c r="N1" s="199"/>
+      <c r="O1" s="199"/>
+      <c r="P1" s="199"/>
+      <c r="Q1" s="199"/>
+      <c r="R1" s="199"/>
+      <c r="S1" s="199"/>
+      <c r="T1" s="199"/>
+      <c r="U1" s="199"/>
+      <c r="V1" s="199"/>
+      <c r="W1" s="199"/>
+      <c r="X1" s="199"/>
     </row>
     <row r="2" spans="1:25" ht="14.25" customHeight="1">
-      <c r="S2" s="62" t="s">
-        <v>222</v>
-      </c>
-      <c r="T2" s="62"/>
-      <c r="U2" s="63"/>
-      <c r="V2" s="63"/>
+      <c r="R2" s="189" t="s">
+        <v>231</v>
+      </c>
+      <c r="S2" s="189"/>
+      <c r="T2" s="189"/>
+      <c r="U2" s="189"/>
+      <c r="V2" s="189"/>
+      <c r="W2" s="189"/>
+      <c r="X2" s="189"/>
     </row>
     <row r="3" spans="1:25" ht="18" customHeight="1">
-      <c r="A3" s="64"/>
-      <c r="B3" s="65" t="s">
+      <c r="A3" s="62"/>
+      <c r="B3" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="66"/>
-      <c r="D3" s="66"/>
-      <c r="E3" s="66"/>
-      <c r="F3" s="66"/>
-      <c r="G3" s="66"/>
-      <c r="H3" s="66"/>
-      <c r="I3" s="66"/>
-      <c r="J3" s="66"/>
-      <c r="K3" s="66"/>
-      <c r="L3" s="66"/>
-      <c r="M3" s="66"/>
-      <c r="N3" s="66"/>
-      <c r="O3" s="67" t="s">
+      <c r="C3" s="64"/>
+      <c r="D3" s="64"/>
+      <c r="E3" s="64"/>
+      <c r="F3" s="64"/>
+      <c r="G3" s="64"/>
+      <c r="H3" s="64"/>
+      <c r="I3" s="64"/>
+      <c r="J3" s="64"/>
+      <c r="K3" s="64"/>
+      <c r="L3" s="64"/>
+      <c r="M3" s="64"/>
+      <c r="N3" s="64"/>
+      <c r="O3" s="65" t="s">
         <v>101</v>
       </c>
-      <c r="P3" s="67"/>
+      <c r="P3" s="65"/>
       <c r="Q3" s="54"/>
-      <c r="R3" s="344" t="s">
+      <c r="R3" s="203" t="s">
         <v>169</v>
       </c>
-      <c r="S3" s="345"/>
-      <c r="T3" s="345"/>
-      <c r="U3" s="345"/>
-      <c r="V3" s="345"/>
-      <c r="W3" s="345"/>
-      <c r="X3" s="346"/>
+      <c r="S3" s="204"/>
+      <c r="T3" s="204"/>
+      <c r="U3" s="204"/>
+      <c r="V3" s="204"/>
+      <c r="W3" s="204"/>
+      <c r="X3" s="205"/>
     </row>
     <row r="4" spans="1:25" ht="12.75" customHeight="1">
-      <c r="A4" s="68"/>
-      <c r="B4" s="69" t="s">
+      <c r="A4" s="66"/>
+      <c r="B4" s="67" t="s">
         <v>5</v>
       </c>
-      <c r="M4" s="70"/>
-      <c r="O4" s="71" t="s">
+      <c r="M4" s="68"/>
+      <c r="O4" s="69" t="s">
         <v>102</v>
       </c>
-      <c r="P4" s="71"/>
+      <c r="P4" s="69"/>
       <c r="Q4"/>
-      <c r="R4" s="347"/>
-      <c r="S4" s="348"/>
-      <c r="T4" s="348"/>
-      <c r="U4" s="348"/>
-      <c r="V4" s="348"/>
-      <c r="W4" s="348"/>
-      <c r="X4" s="349"/>
+      <c r="R4" s="206"/>
+      <c r="S4" s="207"/>
+      <c r="T4" s="207"/>
+      <c r="U4" s="207"/>
+      <c r="V4" s="207"/>
+      <c r="W4" s="207"/>
+      <c r="X4" s="208"/>
     </row>
     <row r="5" spans="1:25" ht="13.5" customHeight="1">
-      <c r="A5" s="68"/>
-      <c r="B5" s="70" t="s">
+      <c r="A5" s="66"/>
+      <c r="B5" s="68" t="s">
         <v>168</v>
       </c>
-      <c r="O5" s="72" t="s">
+      <c r="O5" s="70" t="s">
         <v>103</v>
       </c>
-      <c r="P5" s="72"/>
+      <c r="P5" s="70"/>
       <c r="Q5" s="16"/>
-      <c r="R5" s="350" t="s">
+      <c r="R5" s="209" t="s">
         <v>170</v>
       </c>
-      <c r="S5" s="351"/>
-      <c r="T5" s="351"/>
-      <c r="U5" s="351"/>
-      <c r="V5" s="351"/>
-      <c r="W5" s="351"/>
-      <c r="X5" s="352"/>
+      <c r="S5" s="210"/>
+      <c r="T5" s="210"/>
+      <c r="U5" s="210"/>
+      <c r="V5" s="210"/>
+      <c r="W5" s="210"/>
+      <c r="X5" s="211"/>
     </row>
     <row r="6" spans="1:25" ht="12.75" customHeight="1">
-      <c r="A6" s="73"/>
-      <c r="B6" s="74" t="s">
+      <c r="A6" s="71"/>
+      <c r="B6" s="72" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="75"/>
-      <c r="D6" s="75"/>
-      <c r="E6" s="75"/>
-      <c r="F6" s="75"/>
-      <c r="G6" s="75"/>
-      <c r="H6" s="75"/>
-      <c r="I6" s="75"/>
-      <c r="J6" s="75"/>
-      <c r="K6" s="75"/>
-      <c r="L6" s="75"/>
-      <c r="M6" s="75"/>
-      <c r="N6" s="75"/>
-      <c r="O6" s="76" t="s">
+      <c r="C6" s="73"/>
+      <c r="D6" s="73"/>
+      <c r="E6" s="73"/>
+      <c r="F6" s="73"/>
+      <c r="G6" s="73"/>
+      <c r="H6" s="73"/>
+      <c r="I6" s="73"/>
+      <c r="J6" s="73"/>
+      <c r="K6" s="73"/>
+      <c r="L6" s="73"/>
+      <c r="M6" s="73"/>
+      <c r="N6" s="73"/>
+      <c r="O6" s="74" t="s">
         <v>104</v>
       </c>
-      <c r="P6" s="76"/>
+      <c r="P6" s="74"/>
       <c r="Q6" s="60"/>
-      <c r="R6" s="353"/>
-      <c r="S6" s="354"/>
-      <c r="T6" s="354"/>
-      <c r="U6" s="354"/>
-      <c r="V6" s="354"/>
-      <c r="W6" s="354"/>
-      <c r="X6" s="355"/>
+      <c r="R6" s="212"/>
+      <c r="S6" s="213"/>
+      <c r="T6" s="213"/>
+      <c r="U6" s="213"/>
+      <c r="V6" s="213"/>
+      <c r="W6" s="213"/>
+      <c r="X6" s="214"/>
     </row>
-    <row r="7" spans="1:25" s="80" customFormat="1" ht="5.25" customHeight="1">
-      <c r="A7" s="77"/>
-      <c r="B7" s="78"/>
-      <c r="C7" s="79"/>
-      <c r="E7" s="81"/>
-      <c r="F7" s="79"/>
-      <c r="P7" s="82"/>
-      <c r="Q7" s="83"/>
-      <c r="S7" s="83"/>
-      <c r="T7" s="84"/>
-      <c r="U7" s="85"/>
+    <row r="7" spans="1:25" s="78" customFormat="1" ht="5.25" customHeight="1">
+      <c r="A7" s="75"/>
+      <c r="B7" s="76"/>
+      <c r="C7" s="77"/>
+      <c r="E7" s="79"/>
+      <c r="F7" s="77"/>
+      <c r="P7" s="80"/>
+      <c r="Q7" s="81"/>
+      <c r="S7" s="81"/>
+      <c r="T7" s="82"/>
+      <c r="U7" s="83"/>
       <c r="V7" s="54"/>
-      <c r="W7" s="86"/>
-      <c r="X7" s="87"/>
-      <c r="Y7" s="79"/>
+      <c r="W7" s="84"/>
+      <c r="X7" s="85"/>
+      <c r="Y7" s="77"/>
     </row>
-    <row r="8" spans="1:25" s="100" customFormat="1" ht="69" customHeight="1">
-      <c r="A8" s="88" t="s">
+    <row r="8" spans="1:25" s="98" customFormat="1" ht="69" customHeight="1">
+      <c r="A8" s="86" t="s">
         <v>105</v>
       </c>
-      <c r="B8" s="89" t="s">
+      <c r="B8" s="87" t="s">
         <v>106</v>
       </c>
-      <c r="C8" s="90" t="s">
+      <c r="C8" s="88" t="s">
         <v>107</v>
       </c>
-      <c r="D8" s="91" t="s">
+      <c r="D8" s="89" t="s">
         <v>108</v>
       </c>
-      <c r="E8" s="92" t="s">
+      <c r="E8" s="90" t="s">
         <v>109</v>
       </c>
-      <c r="F8" s="93" t="s">
+      <c r="F8" s="91" t="s">
         <v>110</v>
       </c>
-      <c r="G8" s="91" t="s">
+      <c r="G8" s="89" t="s">
         <v>111</v>
       </c>
-      <c r="H8" s="91" t="s">
+      <c r="H8" s="89" t="s">
         <v>112</v>
       </c>
-      <c r="I8" s="91" t="s">
+      <c r="I8" s="89" t="s">
         <v>113</v>
       </c>
-      <c r="J8" s="91" t="s">
+      <c r="J8" s="89" t="s">
         <v>114</v>
       </c>
-      <c r="K8" s="91" t="s">
+      <c r="K8" s="89" t="s">
         <v>115</v>
       </c>
-      <c r="L8" s="91" t="s">
+      <c r="L8" s="89" t="s">
         <v>116</v>
       </c>
-      <c r="M8" s="91" t="s">
+      <c r="M8" s="89" t="s">
         <v>117</v>
       </c>
-      <c r="N8" s="91" t="s">
+      <c r="N8" s="89" t="s">
         <v>118</v>
       </c>
-      <c r="O8" s="94" t="s">
+      <c r="O8" s="92" t="s">
         <v>119</v>
       </c>
-      <c r="P8" s="91" t="s">
+      <c r="P8" s="89" t="s">
         <v>120</v>
       </c>
-      <c r="Q8" s="91" t="s">
+      <c r="Q8" s="89" t="s">
         <v>121</v>
       </c>
-      <c r="R8" s="91" t="s">
+      <c r="R8" s="89" t="s">
         <v>122</v>
       </c>
-      <c r="S8" s="91" t="s">
+      <c r="S8" s="89" t="s">
         <v>123</v>
       </c>
-      <c r="T8" s="95" t="s">
+      <c r="T8" s="93" t="s">
         <v>124</v>
       </c>
-      <c r="U8" s="96"/>
-      <c r="V8" s="97" t="s">
+      <c r="U8" s="94"/>
+      <c r="V8" s="95" t="s">
         <v>125</v>
       </c>
-      <c r="W8" s="98"/>
-      <c r="X8" s="99" t="s">
+      <c r="W8" s="96"/>
+      <c r="X8" s="97" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="9" spans="1:25" ht="71.25" customHeight="1">
-      <c r="A9" s="101" t="s">
+      <c r="A9" s="99" t="s">
         <v>127</v>
       </c>
-      <c r="B9" s="102" t="s">
+      <c r="B9" s="100" t="s">
         <v>128</v>
       </c>
-      <c r="C9" s="103" t="s">
+      <c r="C9" s="101" t="s">
         <v>129</v>
       </c>
-      <c r="D9" s="104" t="s">
+      <c r="D9" s="102" t="s">
         <v>130</v>
       </c>
-      <c r="E9" s="105" t="s">
+      <c r="E9" s="103" t="s">
         <v>131</v>
       </c>
-      <c r="F9" s="103" t="s">
+      <c r="F9" s="101" t="s">
         <v>132</v>
       </c>
-      <c r="G9" s="104" t="s">
+      <c r="G9" s="102" t="s">
         <v>133</v>
       </c>
-      <c r="H9" s="104" t="s">
+      <c r="H9" s="102" t="s">
         <v>134</v>
       </c>
-      <c r="I9" s="104" t="s">
+      <c r="I9" s="102" t="s">
         <v>135</v>
       </c>
-      <c r="J9" s="104" t="s">
+      <c r="J9" s="102" t="s">
         <v>136</v>
       </c>
-      <c r="K9" s="104" t="s">
+      <c r="K9" s="102" t="s">
         <v>137</v>
       </c>
-      <c r="L9" s="104" t="s">
+      <c r="L9" s="102" t="s">
         <v>138</v>
       </c>
-      <c r="M9" s="104" t="s">
+      <c r="M9" s="102" t="s">
         <v>139</v>
       </c>
-      <c r="N9" s="104" t="s">
+      <c r="N9" s="102" t="s">
         <v>140</v>
       </c>
-      <c r="O9" s="104" t="s">
+      <c r="O9" s="102" t="s">
         <v>141</v>
       </c>
-      <c r="P9" s="104" t="s">
+      <c r="P9" s="102" t="s">
         <v>142</v>
       </c>
-      <c r="Q9" s="104" t="s">
+      <c r="Q9" s="102" t="s">
         <v>143</v>
       </c>
-      <c r="R9" s="104" t="s">
+      <c r="R9" s="102" t="s">
         <v>144</v>
       </c>
-      <c r="S9" s="104" t="s">
+      <c r="S9" s="102" t="s">
         <v>145</v>
       </c>
-      <c r="T9" s="106" t="s">
+      <c r="T9" s="104" t="s">
         <v>146</v>
       </c>
-      <c r="U9" s="107"/>
-      <c r="V9" s="108" t="s">
+      <c r="U9" s="105"/>
+      <c r="V9" s="106" t="s">
         <v>147</v>
       </c>
-      <c r="W9" s="79"/>
-      <c r="X9" s="109" t="s">
+      <c r="W9" s="77"/>
+      <c r="X9" s="107" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="10" spans="1:25" s="100" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A10" s="186"/>
-      <c r="B10" s="110"/>
-      <c r="C10" s="111"/>
-      <c r="D10" s="112"/>
-      <c r="E10" s="110"/>
-      <c r="F10" s="111" t="s">
+    <row r="10" spans="1:25" s="98" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A10" s="184"/>
+      <c r="B10" s="108"/>
+      <c r="C10" s="109"/>
+      <c r="D10" s="110"/>
+      <c r="E10" s="108"/>
+      <c r="F10" s="109" t="s">
         <v>149</v>
       </c>
-      <c r="G10" s="112" t="s">
+      <c r="G10" s="110" t="s">
         <v>150</v>
       </c>
-      <c r="H10" s="112" t="s">
+      <c r="H10" s="110" t="s">
         <v>151</v>
       </c>
-      <c r="I10" s="112" t="s">
+      <c r="I10" s="110" t="s">
         <v>152</v>
       </c>
-      <c r="J10" s="112" t="s">
+      <c r="J10" s="110" t="s">
         <v>153</v>
       </c>
-      <c r="K10" s="112" t="s">
+      <c r="K10" s="110" t="s">
         <v>154</v>
       </c>
-      <c r="L10" s="112" t="s">
+      <c r="L10" s="110" t="s">
         <v>155</v>
       </c>
-      <c r="M10" s="112" t="s">
+      <c r="M10" s="110" t="s">
         <v>156</v>
       </c>
-      <c r="N10" s="112" t="s">
+      <c r="N10" s="110" t="s">
         <v>157</v>
       </c>
-      <c r="O10" s="112" t="s">
+      <c r="O10" s="110" t="s">
         <v>158</v>
       </c>
-      <c r="P10" s="112" t="s">
+      <c r="P10" s="110" t="s">
         <v>159</v>
       </c>
-      <c r="Q10" s="112" t="s">
+      <c r="Q10" s="110" t="s">
         <v>160</v>
       </c>
-      <c r="R10" s="112" t="s">
+      <c r="R10" s="110" t="s">
         <v>161</v>
       </c>
-      <c r="S10" s="112" t="s">
+      <c r="S10" s="110" t="s">
         <v>162</v>
       </c>
-      <c r="T10" s="113" t="s">
+      <c r="T10" s="111" t="s">
         <v>163</v>
       </c>
-      <c r="U10" s="341" t="s">
-        <v>223</v>
-      </c>
-      <c r="V10" s="342"/>
-      <c r="W10" s="343"/>
-      <c r="X10" s="114"/>
+      <c r="U10" s="200" t="s">
+        <v>222</v>
+      </c>
+      <c r="V10" s="201"/>
+      <c r="W10" s="202"/>
+      <c r="X10" s="112"/>
     </row>
     <row r="11" spans="1:25" ht="18.899999999999999" customHeight="1">
-      <c r="A11" s="185"/>
-      <c r="B11" s="164"/>
-      <c r="C11" s="165"/>
-      <c r="D11" s="166"/>
-      <c r="E11" s="167"/>
-      <c r="F11" s="168"/>
-      <c r="G11" s="166"/>
-      <c r="H11" s="166"/>
-      <c r="I11" s="166"/>
-      <c r="J11" s="166"/>
-      <c r="K11" s="166"/>
-      <c r="L11" s="166"/>
-      <c r="M11" s="166"/>
-      <c r="N11" s="166"/>
-      <c r="O11" s="166"/>
-      <c r="P11" s="166"/>
-      <c r="Q11" s="166"/>
-      <c r="R11" s="166"/>
-      <c r="S11" s="166"/>
-      <c r="T11" s="169"/>
-      <c r="U11" s="338"/>
-      <c r="V11" s="339"/>
-      <c r="W11" s="340"/>
-      <c r="X11" s="187"/>
+      <c r="A11" s="183"/>
+      <c r="B11" s="162"/>
+      <c r="C11" s="163"/>
+      <c r="D11" s="164"/>
+      <c r="E11" s="165"/>
+      <c r="F11" s="166"/>
+      <c r="G11" s="164"/>
+      <c r="H11" s="164"/>
+      <c r="I11" s="164"/>
+      <c r="J11" s="164"/>
+      <c r="K11" s="164"/>
+      <c r="L11" s="164"/>
+      <c r="M11" s="164"/>
+      <c r="N11" s="164"/>
+      <c r="O11" s="164"/>
+      <c r="P11" s="164"/>
+      <c r="Q11" s="164"/>
+      <c r="R11" s="164"/>
+      <c r="S11" s="164"/>
+      <c r="T11" s="167"/>
+      <c r="U11" s="196"/>
+      <c r="V11" s="197"/>
+      <c r="W11" s="198"/>
+      <c r="X11" s="185"/>
     </row>
     <row r="12" spans="1:25" ht="18.899999999999999" customHeight="1">
-      <c r="A12" s="170"/>
-      <c r="B12" s="164"/>
-      <c r="C12" s="165"/>
-      <c r="D12" s="171"/>
-      <c r="E12" s="167"/>
-      <c r="F12" s="172"/>
-      <c r="G12" s="173"/>
-      <c r="H12" s="173"/>
-      <c r="I12" s="173"/>
-      <c r="J12" s="173"/>
-      <c r="K12" s="173"/>
-      <c r="L12" s="173"/>
-      <c r="M12" s="173"/>
-      <c r="N12" s="173"/>
-      <c r="O12" s="173"/>
-      <c r="P12" s="173"/>
-      <c r="Q12" s="173"/>
-      <c r="R12" s="173"/>
-      <c r="S12" s="173"/>
-      <c r="T12" s="174"/>
-      <c r="U12" s="332"/>
-      <c r="V12" s="333"/>
-      <c r="W12" s="334"/>
-      <c r="X12" s="188"/>
+      <c r="A12" s="168"/>
+      <c r="B12" s="162"/>
+      <c r="C12" s="163"/>
+      <c r="D12" s="169"/>
+      <c r="E12" s="165"/>
+      <c r="F12" s="170"/>
+      <c r="G12" s="171"/>
+      <c r="H12" s="171"/>
+      <c r="I12" s="171"/>
+      <c r="J12" s="171"/>
+      <c r="K12" s="171"/>
+      <c r="L12" s="171"/>
+      <c r="M12" s="171"/>
+      <c r="N12" s="171"/>
+      <c r="O12" s="171"/>
+      <c r="P12" s="171"/>
+      <c r="Q12" s="171"/>
+      <c r="R12" s="171"/>
+      <c r="S12" s="171"/>
+      <c r="T12" s="172"/>
+      <c r="U12" s="190"/>
+      <c r="V12" s="191"/>
+      <c r="W12" s="192"/>
+      <c r="X12" s="186"/>
     </row>
     <row r="13" spans="1:25" ht="18.899999999999999" customHeight="1">
-      <c r="A13" s="170"/>
-      <c r="B13" s="164"/>
-      <c r="C13" s="165"/>
-      <c r="D13" s="171"/>
-      <c r="E13" s="167"/>
-      <c r="F13" s="168"/>
-      <c r="G13" s="173"/>
-      <c r="H13" s="173"/>
-      <c r="I13" s="173"/>
-      <c r="J13" s="173"/>
-      <c r="K13" s="173"/>
-      <c r="L13" s="173"/>
-      <c r="M13" s="173"/>
-      <c r="N13" s="173"/>
-      <c r="O13" s="173"/>
-      <c r="P13" s="173"/>
-      <c r="Q13" s="173"/>
-      <c r="R13" s="173"/>
-      <c r="S13" s="173"/>
-      <c r="T13" s="174"/>
-      <c r="U13" s="332"/>
-      <c r="V13" s="333"/>
-      <c r="W13" s="334"/>
-      <c r="X13" s="189"/>
+      <c r="A13" s="168"/>
+      <c r="B13" s="162"/>
+      <c r="C13" s="163"/>
+      <c r="D13" s="169"/>
+      <c r="E13" s="165"/>
+      <c r="F13" s="166"/>
+      <c r="G13" s="171"/>
+      <c r="H13" s="171"/>
+      <c r="I13" s="171"/>
+      <c r="J13" s="171"/>
+      <c r="K13" s="171"/>
+      <c r="L13" s="171"/>
+      <c r="M13" s="171"/>
+      <c r="N13" s="171"/>
+      <c r="O13" s="171"/>
+      <c r="P13" s="171"/>
+      <c r="Q13" s="171"/>
+      <c r="R13" s="171"/>
+      <c r="S13" s="171"/>
+      <c r="T13" s="172"/>
+      <c r="U13" s="190"/>
+      <c r="V13" s="191"/>
+      <c r="W13" s="192"/>
+      <c r="X13" s="187"/>
     </row>
     <row r="14" spans="1:25" ht="18.899999999999999" customHeight="1">
-      <c r="A14" s="170"/>
-      <c r="B14" s="164"/>
-      <c r="C14" s="165"/>
-      <c r="D14" s="171"/>
-      <c r="E14" s="167"/>
-      <c r="F14" s="172"/>
-      <c r="G14" s="173"/>
-      <c r="H14" s="173"/>
-      <c r="I14" s="173"/>
-      <c r="J14" s="173"/>
-      <c r="K14" s="173"/>
-      <c r="L14" s="173"/>
-      <c r="M14" s="173"/>
-      <c r="N14" s="173"/>
-      <c r="O14" s="173"/>
-      <c r="P14" s="173"/>
-      <c r="Q14" s="173"/>
-      <c r="R14" s="173"/>
-      <c r="S14" s="173"/>
-      <c r="T14" s="174"/>
-      <c r="U14" s="332"/>
-      <c r="V14" s="333"/>
-      <c r="W14" s="334"/>
-      <c r="X14" s="175"/>
+      <c r="A14" s="168"/>
+      <c r="B14" s="162"/>
+      <c r="C14" s="163"/>
+      <c r="D14" s="169"/>
+      <c r="E14" s="165"/>
+      <c r="F14" s="170"/>
+      <c r="G14" s="171"/>
+      <c r="H14" s="171"/>
+      <c r="I14" s="171"/>
+      <c r="J14" s="171"/>
+      <c r="K14" s="171"/>
+      <c r="L14" s="171"/>
+      <c r="M14" s="171"/>
+      <c r="N14" s="171"/>
+      <c r="O14" s="171"/>
+      <c r="P14" s="171"/>
+      <c r="Q14" s="171"/>
+      <c r="R14" s="171"/>
+      <c r="S14" s="171"/>
+      <c r="T14" s="172"/>
+      <c r="U14" s="190"/>
+      <c r="V14" s="191"/>
+      <c r="W14" s="192"/>
+      <c r="X14" s="173"/>
     </row>
     <row r="15" spans="1:25" ht="18.899999999999999" customHeight="1">
-      <c r="A15" s="170"/>
-      <c r="B15" s="164"/>
-      <c r="C15" s="165"/>
-      <c r="D15" s="171"/>
-      <c r="E15" s="167"/>
-      <c r="F15" s="168"/>
-      <c r="G15" s="173"/>
-      <c r="H15" s="173"/>
-      <c r="I15" s="173"/>
-      <c r="J15" s="173"/>
-      <c r="K15" s="173"/>
-      <c r="L15" s="173"/>
-      <c r="M15" s="173"/>
-      <c r="N15" s="173"/>
-      <c r="O15" s="173"/>
-      <c r="P15" s="173"/>
-      <c r="Q15" s="173"/>
-      <c r="R15" s="173"/>
-      <c r="S15" s="173"/>
-      <c r="T15" s="174"/>
-      <c r="U15" s="332"/>
-      <c r="V15" s="333"/>
-      <c r="W15" s="334"/>
-      <c r="X15" s="175"/>
+      <c r="A15" s="168"/>
+      <c r="B15" s="162"/>
+      <c r="C15" s="163"/>
+      <c r="D15" s="169"/>
+      <c r="E15" s="165"/>
+      <c r="F15" s="166"/>
+      <c r="G15" s="171"/>
+      <c r="H15" s="171"/>
+      <c r="I15" s="171"/>
+      <c r="J15" s="171"/>
+      <c r="K15" s="171"/>
+      <c r="L15" s="171"/>
+      <c r="M15" s="171"/>
+      <c r="N15" s="171"/>
+      <c r="O15" s="171"/>
+      <c r="P15" s="171"/>
+      <c r="Q15" s="171"/>
+      <c r="R15" s="171"/>
+      <c r="S15" s="171"/>
+      <c r="T15" s="172"/>
+      <c r="U15" s="190"/>
+      <c r="V15" s="191"/>
+      <c r="W15" s="192"/>
+      <c r="X15" s="173"/>
     </row>
     <row r="16" spans="1:25" ht="18.899999999999999" customHeight="1">
-      <c r="A16" s="170"/>
-      <c r="B16" s="164"/>
-      <c r="C16" s="165"/>
-      <c r="D16" s="171"/>
-      <c r="E16" s="167"/>
-      <c r="F16" s="172"/>
-      <c r="G16" s="173"/>
-      <c r="H16" s="173"/>
-      <c r="I16" s="173"/>
-      <c r="J16" s="173"/>
-      <c r="K16" s="173"/>
-      <c r="L16" s="173"/>
-      <c r="M16" s="173"/>
-      <c r="N16" s="173"/>
-      <c r="O16" s="173"/>
-      <c r="P16" s="173"/>
-      <c r="Q16" s="173"/>
-      <c r="R16" s="173"/>
-      <c r="S16" s="173"/>
-      <c r="T16" s="174"/>
-      <c r="U16" s="332"/>
-      <c r="V16" s="333"/>
-      <c r="W16" s="334"/>
-      <c r="X16" s="175"/>
+      <c r="A16" s="168"/>
+      <c r="B16" s="162"/>
+      <c r="C16" s="163"/>
+      <c r="D16" s="169"/>
+      <c r="E16" s="165"/>
+      <c r="F16" s="170"/>
+      <c r="G16" s="171"/>
+      <c r="H16" s="171"/>
+      <c r="I16" s="171"/>
+      <c r="J16" s="171"/>
+      <c r="K16" s="171"/>
+      <c r="L16" s="171"/>
+      <c r="M16" s="171"/>
+      <c r="N16" s="171"/>
+      <c r="O16" s="171"/>
+      <c r="P16" s="171"/>
+      <c r="Q16" s="171"/>
+      <c r="R16" s="171"/>
+      <c r="S16" s="171"/>
+      <c r="T16" s="172"/>
+      <c r="U16" s="190"/>
+      <c r="V16" s="191"/>
+      <c r="W16" s="192"/>
+      <c r="X16" s="173"/>
     </row>
     <row r="17" spans="1:24" ht="18.899999999999999" customHeight="1">
-      <c r="A17" s="163"/>
-      <c r="B17" s="164"/>
-      <c r="C17" s="165"/>
-      <c r="D17" s="171"/>
-      <c r="E17" s="167"/>
-      <c r="F17" s="172"/>
-      <c r="G17" s="173"/>
-      <c r="H17" s="173"/>
-      <c r="I17" s="173"/>
-      <c r="J17" s="173"/>
-      <c r="K17" s="173"/>
-      <c r="L17" s="173"/>
-      <c r="M17" s="173"/>
-      <c r="N17" s="173"/>
-      <c r="O17" s="173"/>
-      <c r="P17" s="173"/>
-      <c r="Q17" s="173"/>
-      <c r="R17" s="173"/>
-      <c r="S17" s="173"/>
-      <c r="T17" s="174"/>
-      <c r="U17" s="338"/>
-      <c r="V17" s="339"/>
-      <c r="W17" s="340"/>
-      <c r="X17" s="187"/>
+      <c r="A17" s="161"/>
+      <c r="B17" s="162"/>
+      <c r="C17" s="163"/>
+      <c r="D17" s="169"/>
+      <c r="E17" s="165"/>
+      <c r="F17" s="170"/>
+      <c r="G17" s="171"/>
+      <c r="H17" s="171"/>
+      <c r="I17" s="171"/>
+      <c r="J17" s="171"/>
+      <c r="K17" s="171"/>
+      <c r="L17" s="171"/>
+      <c r="M17" s="171"/>
+      <c r="N17" s="171"/>
+      <c r="O17" s="171"/>
+      <c r="P17" s="171"/>
+      <c r="Q17" s="171"/>
+      <c r="R17" s="171"/>
+      <c r="S17" s="171"/>
+      <c r="T17" s="172"/>
+      <c r="U17" s="196"/>
+      <c r="V17" s="197"/>
+      <c r="W17" s="198"/>
+      <c r="X17" s="185"/>
     </row>
     <row r="18" spans="1:24" ht="18.899999999999999" customHeight="1">
-      <c r="A18" s="185"/>
-      <c r="B18" s="164"/>
-      <c r="C18" s="165"/>
-      <c r="D18" s="171"/>
-      <c r="E18" s="167"/>
-      <c r="F18" s="168"/>
-      <c r="G18" s="173"/>
-      <c r="H18" s="173"/>
-      <c r="I18" s="173"/>
-      <c r="J18" s="173"/>
-      <c r="K18" s="173"/>
-      <c r="L18" s="173"/>
-      <c r="M18" s="173"/>
-      <c r="N18" s="173"/>
-      <c r="O18" s="173"/>
-      <c r="P18" s="173"/>
-      <c r="Q18" s="173"/>
-      <c r="R18" s="173"/>
-      <c r="S18" s="173"/>
-      <c r="T18" s="174"/>
-      <c r="U18" s="338"/>
-      <c r="V18" s="339"/>
-      <c r="W18" s="340"/>
-      <c r="X18" s="187"/>
+      <c r="A18" s="183"/>
+      <c r="B18" s="162"/>
+      <c r="C18" s="163"/>
+      <c r="D18" s="169"/>
+      <c r="E18" s="165"/>
+      <c r="F18" s="166"/>
+      <c r="G18" s="171"/>
+      <c r="H18" s="171"/>
+      <c r="I18" s="171"/>
+      <c r="J18" s="171"/>
+      <c r="K18" s="171"/>
+      <c r="L18" s="171"/>
+      <c r="M18" s="171"/>
+      <c r="N18" s="171"/>
+      <c r="O18" s="171"/>
+      <c r="P18" s="171"/>
+      <c r="Q18" s="171"/>
+      <c r="R18" s="171"/>
+      <c r="S18" s="171"/>
+      <c r="T18" s="172"/>
+      <c r="U18" s="196"/>
+      <c r="V18" s="197"/>
+      <c r="W18" s="198"/>
+      <c r="X18" s="185"/>
     </row>
     <row r="19" spans="1:24" ht="18.899999999999999" customHeight="1">
-      <c r="A19" s="170"/>
-      <c r="B19" s="164"/>
-      <c r="C19" s="165"/>
-      <c r="D19" s="171"/>
-      <c r="E19" s="167"/>
-      <c r="F19" s="172"/>
-      <c r="G19" s="173"/>
-      <c r="H19" s="173"/>
-      <c r="I19" s="173"/>
-      <c r="J19" s="173"/>
-      <c r="K19" s="173"/>
-      <c r="L19" s="173"/>
-      <c r="M19" s="173"/>
-      <c r="N19" s="173"/>
-      <c r="O19" s="173"/>
-      <c r="P19" s="173"/>
-      <c r="Q19" s="173"/>
-      <c r="R19" s="173"/>
-      <c r="S19" s="173"/>
-      <c r="T19" s="174"/>
-      <c r="U19" s="332"/>
-      <c r="V19" s="333"/>
-      <c r="W19" s="334"/>
-      <c r="X19" s="190"/>
+      <c r="A19" s="168"/>
+      <c r="B19" s="162"/>
+      <c r="C19" s="163"/>
+      <c r="D19" s="169"/>
+      <c r="E19" s="165"/>
+      <c r="F19" s="170"/>
+      <c r="G19" s="171"/>
+      <c r="H19" s="171"/>
+      <c r="I19" s="171"/>
+      <c r="J19" s="171"/>
+      <c r="K19" s="171"/>
+      <c r="L19" s="171"/>
+      <c r="M19" s="171"/>
+      <c r="N19" s="171"/>
+      <c r="O19" s="171"/>
+      <c r="P19" s="171"/>
+      <c r="Q19" s="171"/>
+      <c r="R19" s="171"/>
+      <c r="S19" s="171"/>
+      <c r="T19" s="172"/>
+      <c r="U19" s="190"/>
+      <c r="V19" s="191"/>
+      <c r="W19" s="192"/>
+      <c r="X19" s="188"/>
     </row>
     <row r="20" spans="1:24" ht="18.899999999999999" customHeight="1">
-      <c r="A20" s="170"/>
-      <c r="B20" s="164"/>
-      <c r="C20" s="165"/>
-      <c r="D20" s="171"/>
-      <c r="E20" s="167"/>
-      <c r="F20" s="172"/>
-      <c r="G20" s="173"/>
-      <c r="H20" s="173"/>
-      <c r="I20" s="173"/>
-      <c r="J20" s="173"/>
-      <c r="K20" s="173"/>
-      <c r="L20" s="173"/>
-      <c r="M20" s="173"/>
-      <c r="N20" s="173"/>
-      <c r="O20" s="173"/>
-      <c r="P20" s="173"/>
-      <c r="Q20" s="173"/>
-      <c r="R20" s="173"/>
-      <c r="S20" s="173"/>
-      <c r="T20" s="174"/>
-      <c r="U20" s="338"/>
-      <c r="V20" s="339"/>
-      <c r="W20" s="340"/>
-      <c r="X20" s="187"/>
+      <c r="A20" s="168"/>
+      <c r="B20" s="162"/>
+      <c r="C20" s="163"/>
+      <c r="D20" s="169"/>
+      <c r="E20" s="165"/>
+      <c r="F20" s="170"/>
+      <c r="G20" s="171"/>
+      <c r="H20" s="171"/>
+      <c r="I20" s="171"/>
+      <c r="J20" s="171"/>
+      <c r="K20" s="171"/>
+      <c r="L20" s="171"/>
+      <c r="M20" s="171"/>
+      <c r="N20" s="171"/>
+      <c r="O20" s="171"/>
+      <c r="P20" s="171"/>
+      <c r="Q20" s="171"/>
+      <c r="R20" s="171"/>
+      <c r="S20" s="171"/>
+      <c r="T20" s="172"/>
+      <c r="U20" s="196"/>
+      <c r="V20" s="197"/>
+      <c r="W20" s="198"/>
+      <c r="X20" s="185"/>
     </row>
     <row r="21" spans="1:24" ht="18.899999999999999" customHeight="1">
-      <c r="A21" s="170"/>
-      <c r="B21" s="164"/>
-      <c r="C21" s="165"/>
-      <c r="D21" s="171"/>
-      <c r="E21" s="167"/>
-      <c r="F21" s="168"/>
-      <c r="G21" s="173"/>
-      <c r="H21" s="173"/>
-      <c r="I21" s="173"/>
-      <c r="J21" s="173"/>
-      <c r="K21" s="173"/>
-      <c r="L21" s="173"/>
-      <c r="M21" s="173"/>
-      <c r="N21" s="173"/>
-      <c r="O21" s="173"/>
-      <c r="P21" s="173"/>
-      <c r="Q21" s="173"/>
-      <c r="R21" s="173"/>
-      <c r="S21" s="173"/>
-      <c r="T21" s="174"/>
-      <c r="U21" s="338"/>
-      <c r="V21" s="339"/>
-      <c r="W21" s="340"/>
-      <c r="X21" s="187"/>
+      <c r="A21" s="168"/>
+      <c r="B21" s="162"/>
+      <c r="C21" s="163"/>
+      <c r="D21" s="169"/>
+      <c r="E21" s="165"/>
+      <c r="F21" s="166"/>
+      <c r="G21" s="171"/>
+      <c r="H21" s="171"/>
+      <c r="I21" s="171"/>
+      <c r="J21" s="171"/>
+      <c r="K21" s="171"/>
+      <c r="L21" s="171"/>
+      <c r="M21" s="171"/>
+      <c r="N21" s="171"/>
+      <c r="O21" s="171"/>
+      <c r="P21" s="171"/>
+      <c r="Q21" s="171"/>
+      <c r="R21" s="171"/>
+      <c r="S21" s="171"/>
+      <c r="T21" s="172"/>
+      <c r="U21" s="196"/>
+      <c r="V21" s="197"/>
+      <c r="W21" s="198"/>
+      <c r="X21" s="185"/>
     </row>
     <row r="22" spans="1:24" ht="18.899999999999999" customHeight="1">
-      <c r="A22" s="170"/>
-      <c r="B22" s="164"/>
-      <c r="C22" s="165"/>
-      <c r="D22" s="171"/>
-      <c r="E22" s="167"/>
-      <c r="F22" s="172"/>
-      <c r="G22" s="173"/>
-      <c r="H22" s="173"/>
-      <c r="I22" s="173"/>
-      <c r="J22" s="173"/>
-      <c r="K22" s="173"/>
-      <c r="L22" s="173"/>
-      <c r="M22" s="173"/>
-      <c r="N22" s="173"/>
-      <c r="O22" s="173"/>
-      <c r="P22" s="173"/>
-      <c r="Q22" s="173"/>
-      <c r="R22" s="173"/>
-      <c r="S22" s="173"/>
-      <c r="T22" s="174"/>
-      <c r="U22" s="332"/>
-      <c r="V22" s="333"/>
-      <c r="W22" s="334"/>
-      <c r="X22" s="188"/>
+      <c r="A22" s="168"/>
+      <c r="B22" s="162"/>
+      <c r="C22" s="163"/>
+      <c r="D22" s="169"/>
+      <c r="E22" s="165"/>
+      <c r="F22" s="170"/>
+      <c r="G22" s="171"/>
+      <c r="H22" s="171"/>
+      <c r="I22" s="171"/>
+      <c r="J22" s="171"/>
+      <c r="K22" s="171"/>
+      <c r="L22" s="171"/>
+      <c r="M22" s="171"/>
+      <c r="N22" s="171"/>
+      <c r="O22" s="171"/>
+      <c r="P22" s="171"/>
+      <c r="Q22" s="171"/>
+      <c r="R22" s="171"/>
+      <c r="S22" s="171"/>
+      <c r="T22" s="172"/>
+      <c r="U22" s="190"/>
+      <c r="V22" s="191"/>
+      <c r="W22" s="192"/>
+      <c r="X22" s="186"/>
     </row>
     <row r="23" spans="1:24" ht="18.899999999999999" customHeight="1">
-      <c r="A23" s="170"/>
-      <c r="B23" s="164"/>
-      <c r="C23" s="165"/>
-      <c r="D23" s="171"/>
-      <c r="E23" s="167"/>
-      <c r="F23" s="172"/>
-      <c r="G23" s="173"/>
-      <c r="H23" s="173"/>
-      <c r="I23" s="173"/>
-      <c r="J23" s="173"/>
-      <c r="K23" s="173"/>
-      <c r="L23" s="173"/>
-      <c r="M23" s="173"/>
-      <c r="N23" s="173"/>
-      <c r="O23" s="173"/>
-      <c r="P23" s="173"/>
-      <c r="Q23" s="173"/>
-      <c r="R23" s="173"/>
-      <c r="S23" s="173"/>
-      <c r="T23" s="174"/>
-      <c r="U23" s="338"/>
-      <c r="V23" s="339"/>
-      <c r="W23" s="340"/>
-      <c r="X23" s="187"/>
+      <c r="A23" s="168"/>
+      <c r="B23" s="162"/>
+      <c r="C23" s="163"/>
+      <c r="D23" s="169"/>
+      <c r="E23" s="165"/>
+      <c r="F23" s="170"/>
+      <c r="G23" s="171"/>
+      <c r="H23" s="171"/>
+      <c r="I23" s="171"/>
+      <c r="J23" s="171"/>
+      <c r="K23" s="171"/>
+      <c r="L23" s="171"/>
+      <c r="M23" s="171"/>
+      <c r="N23" s="171"/>
+      <c r="O23" s="171"/>
+      <c r="P23" s="171"/>
+      <c r="Q23" s="171"/>
+      <c r="R23" s="171"/>
+      <c r="S23" s="171"/>
+      <c r="T23" s="172"/>
+      <c r="U23" s="196"/>
+      <c r="V23" s="197"/>
+      <c r="W23" s="198"/>
+      <c r="X23" s="185"/>
     </row>
     <row r="24" spans="1:24" ht="18.899999999999999" customHeight="1">
-      <c r="A24" s="163"/>
-      <c r="B24" s="164"/>
-      <c r="C24" s="165"/>
-      <c r="D24" s="171"/>
-      <c r="E24" s="167"/>
-      <c r="F24" s="168"/>
-      <c r="G24" s="173"/>
-      <c r="H24" s="173"/>
-      <c r="I24" s="173"/>
-      <c r="J24" s="173"/>
-      <c r="K24" s="173"/>
-      <c r="L24" s="173"/>
-      <c r="M24" s="173"/>
-      <c r="N24" s="173"/>
-      <c r="O24" s="173"/>
-      <c r="P24" s="173"/>
-      <c r="Q24" s="173"/>
-      <c r="R24" s="173"/>
-      <c r="S24" s="173"/>
-      <c r="T24" s="174"/>
-      <c r="U24" s="338"/>
-      <c r="V24" s="339"/>
-      <c r="W24" s="340"/>
-      <c r="X24" s="187"/>
+      <c r="A24" s="161"/>
+      <c r="B24" s="162"/>
+      <c r="C24" s="163"/>
+      <c r="D24" s="169"/>
+      <c r="E24" s="165"/>
+      <c r="F24" s="166"/>
+      <c r="G24" s="171"/>
+      <c r="H24" s="171"/>
+      <c r="I24" s="171"/>
+      <c r="J24" s="171"/>
+      <c r="K24" s="171"/>
+      <c r="L24" s="171"/>
+      <c r="M24" s="171"/>
+      <c r="N24" s="171"/>
+      <c r="O24" s="171"/>
+      <c r="P24" s="171"/>
+      <c r="Q24" s="171"/>
+      <c r="R24" s="171"/>
+      <c r="S24" s="171"/>
+      <c r="T24" s="172"/>
+      <c r="U24" s="196"/>
+      <c r="V24" s="197"/>
+      <c r="W24" s="198"/>
+      <c r="X24" s="185"/>
     </row>
     <row r="25" spans="1:24" ht="18.899999999999999" customHeight="1">
-      <c r="A25" s="185"/>
-      <c r="B25" s="164"/>
-      <c r="C25" s="165"/>
-      <c r="D25" s="171"/>
-      <c r="E25" s="167"/>
-      <c r="F25" s="172"/>
-      <c r="G25" s="173"/>
-      <c r="H25" s="173"/>
-      <c r="I25" s="173"/>
-      <c r="J25" s="173"/>
-      <c r="K25" s="173"/>
-      <c r="L25" s="173"/>
-      <c r="M25" s="173"/>
-      <c r="N25" s="173"/>
-      <c r="O25" s="173"/>
-      <c r="P25" s="173"/>
-      <c r="Q25" s="173"/>
-      <c r="R25" s="173"/>
-      <c r="S25" s="173"/>
-      <c r="T25" s="174"/>
-      <c r="U25" s="338"/>
-      <c r="V25" s="339"/>
-      <c r="W25" s="340"/>
-      <c r="X25" s="187"/>
+      <c r="A25" s="183"/>
+      <c r="B25" s="162"/>
+      <c r="C25" s="163"/>
+      <c r="D25" s="169"/>
+      <c r="E25" s="165"/>
+      <c r="F25" s="170"/>
+      <c r="G25" s="171"/>
+      <c r="H25" s="171"/>
+      <c r="I25" s="171"/>
+      <c r="J25" s="171"/>
+      <c r="K25" s="171"/>
+      <c r="L25" s="171"/>
+      <c r="M25" s="171"/>
+      <c r="N25" s="171"/>
+      <c r="O25" s="171"/>
+      <c r="P25" s="171"/>
+      <c r="Q25" s="171"/>
+      <c r="R25" s="171"/>
+      <c r="S25" s="171"/>
+      <c r="T25" s="172"/>
+      <c r="U25" s="196"/>
+      <c r="V25" s="197"/>
+      <c r="W25" s="198"/>
+      <c r="X25" s="185"/>
     </row>
     <row r="26" spans="1:24" ht="18.899999999999999" customHeight="1">
-      <c r="A26" s="170"/>
-      <c r="B26" s="164"/>
-      <c r="C26" s="165"/>
-      <c r="D26" s="171"/>
-      <c r="E26" s="167"/>
-      <c r="F26" s="172"/>
-      <c r="G26" s="173"/>
-      <c r="H26" s="173"/>
-      <c r="I26" s="173"/>
-      <c r="J26" s="173"/>
-      <c r="K26" s="173"/>
-      <c r="L26" s="173"/>
-      <c r="M26" s="173"/>
-      <c r="N26" s="173"/>
-      <c r="O26" s="173"/>
-      <c r="P26" s="173"/>
-      <c r="Q26" s="173"/>
-      <c r="R26" s="173"/>
-      <c r="S26" s="173"/>
-      <c r="T26" s="174"/>
-      <c r="U26" s="332"/>
-      <c r="V26" s="333"/>
-      <c r="W26" s="334"/>
-      <c r="X26" s="190"/>
+      <c r="A26" s="168"/>
+      <c r="B26" s="162"/>
+      <c r="C26" s="163"/>
+      <c r="D26" s="169"/>
+      <c r="E26" s="165"/>
+      <c r="F26" s="170"/>
+      <c r="G26" s="171"/>
+      <c r="H26" s="171"/>
+      <c r="I26" s="171"/>
+      <c r="J26" s="171"/>
+      <c r="K26" s="171"/>
+      <c r="L26" s="171"/>
+      <c r="M26" s="171"/>
+      <c r="N26" s="171"/>
+      <c r="O26" s="171"/>
+      <c r="P26" s="171"/>
+      <c r="Q26" s="171"/>
+      <c r="R26" s="171"/>
+      <c r="S26" s="171"/>
+      <c r="T26" s="172"/>
+      <c r="U26" s="190"/>
+      <c r="V26" s="191"/>
+      <c r="W26" s="192"/>
+      <c r="X26" s="188"/>
     </row>
     <row r="27" spans="1:24" ht="18.899999999999999" customHeight="1">
-      <c r="A27" s="170"/>
-      <c r="B27" s="164"/>
-      <c r="C27" s="165"/>
-      <c r="D27" s="171"/>
-      <c r="E27" s="167"/>
-      <c r="F27" s="168"/>
-      <c r="G27" s="173"/>
-      <c r="H27" s="173"/>
-      <c r="I27" s="173"/>
-      <c r="J27" s="173"/>
-      <c r="K27" s="173"/>
-      <c r="L27" s="173"/>
-      <c r="M27" s="173"/>
-      <c r="N27" s="173"/>
-      <c r="O27" s="173"/>
-      <c r="P27" s="173"/>
-      <c r="Q27" s="173"/>
-      <c r="R27" s="173"/>
-      <c r="S27" s="173"/>
-      <c r="T27" s="174"/>
-      <c r="U27" s="338"/>
-      <c r="V27" s="339"/>
-      <c r="W27" s="340"/>
-      <c r="X27" s="187"/>
+      <c r="A27" s="168"/>
+      <c r="B27" s="162"/>
+      <c r="C27" s="163"/>
+      <c r="D27" s="169"/>
+      <c r="E27" s="165"/>
+      <c r="F27" s="166"/>
+      <c r="G27" s="171"/>
+      <c r="H27" s="171"/>
+      <c r="I27" s="171"/>
+      <c r="J27" s="171"/>
+      <c r="K27" s="171"/>
+      <c r="L27" s="171"/>
+      <c r="M27" s="171"/>
+      <c r="N27" s="171"/>
+      <c r="O27" s="171"/>
+      <c r="P27" s="171"/>
+      <c r="Q27" s="171"/>
+      <c r="R27" s="171"/>
+      <c r="S27" s="171"/>
+      <c r="T27" s="172"/>
+      <c r="U27" s="196"/>
+      <c r="V27" s="197"/>
+      <c r="W27" s="198"/>
+      <c r="X27" s="185"/>
     </row>
     <row r="28" spans="1:24" ht="18.899999999999999" customHeight="1">
-      <c r="A28" s="170"/>
-      <c r="B28" s="164"/>
-      <c r="C28" s="165"/>
-      <c r="D28" s="171"/>
-      <c r="E28" s="167"/>
-      <c r="F28" s="172"/>
-      <c r="G28" s="173"/>
-      <c r="H28" s="173"/>
-      <c r="I28" s="173"/>
-      <c r="J28" s="173"/>
-      <c r="K28" s="173"/>
-      <c r="L28" s="173"/>
-      <c r="M28" s="173"/>
-      <c r="N28" s="173"/>
-      <c r="O28" s="173"/>
-      <c r="P28" s="173"/>
-      <c r="Q28" s="173"/>
-      <c r="R28" s="173"/>
-      <c r="S28" s="173"/>
-      <c r="T28" s="174"/>
-      <c r="U28" s="332"/>
-      <c r="V28" s="333"/>
-      <c r="W28" s="334"/>
-      <c r="X28" s="188"/>
+      <c r="A28" s="168"/>
+      <c r="B28" s="162"/>
+      <c r="C28" s="163"/>
+      <c r="D28" s="169"/>
+      <c r="E28" s="165"/>
+      <c r="F28" s="170"/>
+      <c r="G28" s="171"/>
+      <c r="H28" s="171"/>
+      <c r="I28" s="171"/>
+      <c r="J28" s="171"/>
+      <c r="K28" s="171"/>
+      <c r="L28" s="171"/>
+      <c r="M28" s="171"/>
+      <c r="N28" s="171"/>
+      <c r="O28" s="171"/>
+      <c r="P28" s="171"/>
+      <c r="Q28" s="171"/>
+      <c r="R28" s="171"/>
+      <c r="S28" s="171"/>
+      <c r="T28" s="172"/>
+      <c r="U28" s="190"/>
+      <c r="V28" s="191"/>
+      <c r="W28" s="192"/>
+      <c r="X28" s="186"/>
     </row>
     <row r="29" spans="1:24" ht="18.899999999999999" customHeight="1">
-      <c r="A29" s="170"/>
-      <c r="B29" s="164"/>
-      <c r="C29" s="165"/>
-      <c r="D29" s="171"/>
-      <c r="E29" s="167"/>
-      <c r="F29" s="172"/>
-      <c r="G29" s="173"/>
-      <c r="H29" s="173"/>
-      <c r="I29" s="173"/>
-      <c r="J29" s="173"/>
-      <c r="K29" s="173"/>
-      <c r="L29" s="173"/>
-      <c r="M29" s="173"/>
-      <c r="N29" s="173"/>
-      <c r="O29" s="173"/>
-      <c r="P29" s="173"/>
-      <c r="Q29" s="173"/>
-      <c r="R29" s="173"/>
-      <c r="S29" s="173"/>
-      <c r="T29" s="174"/>
-      <c r="U29" s="338"/>
-      <c r="V29" s="339"/>
-      <c r="W29" s="340"/>
-      <c r="X29" s="187"/>
+      <c r="A29" s="168"/>
+      <c r="B29" s="162"/>
+      <c r="C29" s="163"/>
+      <c r="D29" s="169"/>
+      <c r="E29" s="165"/>
+      <c r="F29" s="170"/>
+      <c r="G29" s="171"/>
+      <c r="H29" s="171"/>
+      <c r="I29" s="171"/>
+      <c r="J29" s="171"/>
+      <c r="K29" s="171"/>
+      <c r="L29" s="171"/>
+      <c r="M29" s="171"/>
+      <c r="N29" s="171"/>
+      <c r="O29" s="171"/>
+      <c r="P29" s="171"/>
+      <c r="Q29" s="171"/>
+      <c r="R29" s="171"/>
+      <c r="S29" s="171"/>
+      <c r="T29" s="172"/>
+      <c r="U29" s="196"/>
+      <c r="V29" s="197"/>
+      <c r="W29" s="198"/>
+      <c r="X29" s="185"/>
     </row>
     <row r="30" spans="1:24" ht="18.899999999999999" customHeight="1">
-      <c r="A30" s="170"/>
-      <c r="B30" s="164"/>
-      <c r="C30" s="165"/>
-      <c r="D30" s="171"/>
-      <c r="E30" s="167"/>
-      <c r="F30" s="168"/>
-      <c r="G30" s="173"/>
-      <c r="H30" s="173"/>
-      <c r="I30" s="173"/>
-      <c r="J30" s="173"/>
-      <c r="K30" s="173"/>
-      <c r="L30" s="173"/>
-      <c r="M30" s="173"/>
-      <c r="N30" s="173"/>
-      <c r="O30" s="173"/>
-      <c r="P30" s="173"/>
-      <c r="Q30" s="173"/>
-      <c r="R30" s="173"/>
-      <c r="S30" s="173"/>
-      <c r="T30" s="174"/>
-      <c r="U30" s="338"/>
-      <c r="V30" s="339"/>
-      <c r="W30" s="340"/>
-      <c r="X30" s="187"/>
+      <c r="A30" s="168"/>
+      <c r="B30" s="162"/>
+      <c r="C30" s="163"/>
+      <c r="D30" s="169"/>
+      <c r="E30" s="165"/>
+      <c r="F30" s="166"/>
+      <c r="G30" s="171"/>
+      <c r="H30" s="171"/>
+      <c r="I30" s="171"/>
+      <c r="J30" s="171"/>
+      <c r="K30" s="171"/>
+      <c r="L30" s="171"/>
+      <c r="M30" s="171"/>
+      <c r="N30" s="171"/>
+      <c r="O30" s="171"/>
+      <c r="P30" s="171"/>
+      <c r="Q30" s="171"/>
+      <c r="R30" s="171"/>
+      <c r="S30" s="171"/>
+      <c r="T30" s="172"/>
+      <c r="U30" s="196"/>
+      <c r="V30" s="197"/>
+      <c r="W30" s="198"/>
+      <c r="X30" s="185"/>
     </row>
     <row r="31" spans="1:24" ht="18.899999999999999" customHeight="1">
-      <c r="A31" s="163"/>
-      <c r="B31" s="164"/>
-      <c r="C31" s="165"/>
-      <c r="D31" s="171"/>
-      <c r="E31" s="167"/>
-      <c r="F31" s="172"/>
-      <c r="G31" s="173"/>
-      <c r="H31" s="173"/>
-      <c r="I31" s="173"/>
-      <c r="J31" s="173"/>
-      <c r="K31" s="173"/>
-      <c r="L31" s="173"/>
-      <c r="M31" s="173"/>
-      <c r="N31" s="173"/>
-      <c r="O31" s="173"/>
-      <c r="P31" s="173"/>
-      <c r="Q31" s="173"/>
-      <c r="R31" s="173"/>
-      <c r="S31" s="173"/>
-      <c r="T31" s="174"/>
-      <c r="U31" s="332"/>
-      <c r="V31" s="333"/>
-      <c r="W31" s="334"/>
-      <c r="X31" s="188"/>
+      <c r="A31" s="161"/>
+      <c r="B31" s="162"/>
+      <c r="C31" s="163"/>
+      <c r="D31" s="169"/>
+      <c r="E31" s="165"/>
+      <c r="F31" s="170"/>
+      <c r="G31" s="171"/>
+      <c r="H31" s="171"/>
+      <c r="I31" s="171"/>
+      <c r="J31" s="171"/>
+      <c r="K31" s="171"/>
+      <c r="L31" s="171"/>
+      <c r="M31" s="171"/>
+      <c r="N31" s="171"/>
+      <c r="O31" s="171"/>
+      <c r="P31" s="171"/>
+      <c r="Q31" s="171"/>
+      <c r="R31" s="171"/>
+      <c r="S31" s="171"/>
+      <c r="T31" s="172"/>
+      <c r="U31" s="190"/>
+      <c r="V31" s="191"/>
+      <c r="W31" s="192"/>
+      <c r="X31" s="186"/>
     </row>
     <row r="32" spans="1:24" ht="18.899999999999999" customHeight="1">
-      <c r="A32" s="185"/>
-      <c r="B32" s="164"/>
-      <c r="C32" s="165"/>
-      <c r="D32" s="171"/>
-      <c r="E32" s="167"/>
-      <c r="F32" s="172"/>
-      <c r="G32" s="173"/>
-      <c r="H32" s="173"/>
-      <c r="I32" s="173"/>
-      <c r="J32" s="173"/>
-      <c r="K32" s="173"/>
-      <c r="L32" s="173"/>
-      <c r="M32" s="173"/>
-      <c r="N32" s="173"/>
-      <c r="O32" s="173"/>
-      <c r="P32" s="173"/>
-      <c r="Q32" s="173"/>
-      <c r="R32" s="173"/>
-      <c r="S32" s="173"/>
-      <c r="T32" s="174"/>
-      <c r="U32" s="338"/>
-      <c r="V32" s="339"/>
-      <c r="W32" s="340"/>
-      <c r="X32" s="187"/>
+      <c r="A32" s="183"/>
+      <c r="B32" s="162"/>
+      <c r="C32" s="163"/>
+      <c r="D32" s="169"/>
+      <c r="E32" s="165"/>
+      <c r="F32" s="170"/>
+      <c r="G32" s="171"/>
+      <c r="H32" s="171"/>
+      <c r="I32" s="171"/>
+      <c r="J32" s="171"/>
+      <c r="K32" s="171"/>
+      <c r="L32" s="171"/>
+      <c r="M32" s="171"/>
+      <c r="N32" s="171"/>
+      <c r="O32" s="171"/>
+      <c r="P32" s="171"/>
+      <c r="Q32" s="171"/>
+      <c r="R32" s="171"/>
+      <c r="S32" s="171"/>
+      <c r="T32" s="172"/>
+      <c r="U32" s="196"/>
+      <c r="V32" s="197"/>
+      <c r="W32" s="198"/>
+      <c r="X32" s="185"/>
     </row>
     <row r="33" spans="1:24" ht="18.899999999999999" customHeight="1">
-      <c r="A33" s="170"/>
-      <c r="B33" s="164"/>
-      <c r="C33" s="165"/>
-      <c r="D33" s="171"/>
-      <c r="E33" s="167"/>
-      <c r="F33" s="168"/>
-      <c r="G33" s="173"/>
-      <c r="H33" s="173"/>
-      <c r="I33" s="173"/>
-      <c r="J33" s="173"/>
-      <c r="K33" s="173"/>
-      <c r="L33" s="173"/>
-      <c r="M33" s="173"/>
-      <c r="N33" s="173"/>
-      <c r="O33" s="173"/>
-      <c r="P33" s="173"/>
-      <c r="Q33" s="173"/>
-      <c r="R33" s="173"/>
-      <c r="S33" s="173"/>
-      <c r="T33" s="174"/>
-      <c r="U33" s="338"/>
-      <c r="V33" s="339"/>
-      <c r="W33" s="340"/>
-      <c r="X33" s="187"/>
+      <c r="A33" s="168"/>
+      <c r="B33" s="162"/>
+      <c r="C33" s="163"/>
+      <c r="D33" s="169"/>
+      <c r="E33" s="165"/>
+      <c r="F33" s="166"/>
+      <c r="G33" s="171"/>
+      <c r="H33" s="171"/>
+      <c r="I33" s="171"/>
+      <c r="J33" s="171"/>
+      <c r="K33" s="171"/>
+      <c r="L33" s="171"/>
+      <c r="M33" s="171"/>
+      <c r="N33" s="171"/>
+      <c r="O33" s="171"/>
+      <c r="P33" s="171"/>
+      <c r="Q33" s="171"/>
+      <c r="R33" s="171"/>
+      <c r="S33" s="171"/>
+      <c r="T33" s="172"/>
+      <c r="U33" s="196"/>
+      <c r="V33" s="197"/>
+      <c r="W33" s="198"/>
+      <c r="X33" s="185"/>
     </row>
     <row r="34" spans="1:24" ht="18.899999999999999" customHeight="1">
-      <c r="A34" s="170"/>
-      <c r="B34" s="164"/>
-      <c r="C34" s="165"/>
-      <c r="D34" s="171"/>
-      <c r="E34" s="167"/>
-      <c r="F34" s="172"/>
-      <c r="G34" s="173"/>
-      <c r="H34" s="173"/>
-      <c r="I34" s="173"/>
-      <c r="J34" s="173"/>
-      <c r="K34" s="173"/>
-      <c r="L34" s="173"/>
-      <c r="M34" s="173"/>
-      <c r="N34" s="173"/>
-      <c r="O34" s="173"/>
-      <c r="P34" s="173"/>
-      <c r="Q34" s="173"/>
-      <c r="R34" s="173"/>
-      <c r="S34" s="173"/>
-      <c r="T34" s="174"/>
-      <c r="U34" s="332"/>
-      <c r="V34" s="333"/>
-      <c r="W34" s="334"/>
-      <c r="X34" s="188"/>
+      <c r="A34" s="168"/>
+      <c r="B34" s="162"/>
+      <c r="C34" s="163"/>
+      <c r="D34" s="169"/>
+      <c r="E34" s="165"/>
+      <c r="F34" s="170"/>
+      <c r="G34" s="171"/>
+      <c r="H34" s="171"/>
+      <c r="I34" s="171"/>
+      <c r="J34" s="171"/>
+      <c r="K34" s="171"/>
+      <c r="L34" s="171"/>
+      <c r="M34" s="171"/>
+      <c r="N34" s="171"/>
+      <c r="O34" s="171"/>
+      <c r="P34" s="171"/>
+      <c r="Q34" s="171"/>
+      <c r="R34" s="171"/>
+      <c r="S34" s="171"/>
+      <c r="T34" s="172"/>
+      <c r="U34" s="190"/>
+      <c r="V34" s="191"/>
+      <c r="W34" s="192"/>
+      <c r="X34" s="186"/>
     </row>
     <row r="35" spans="1:24" ht="18.899999999999999" customHeight="1">
-      <c r="A35" s="335" t="s">
+      <c r="A35" s="193" t="s">
         <v>199</v>
       </c>
-      <c r="B35" s="336"/>
-      <c r="C35" s="336"/>
-      <c r="D35" s="336"/>
-      <c r="E35" s="336"/>
-      <c r="F35" s="336"/>
-      <c r="G35" s="336"/>
-      <c r="H35" s="336"/>
-      <c r="I35" s="336"/>
-      <c r="J35" s="336"/>
-      <c r="K35" s="336"/>
-      <c r="L35" s="336"/>
-      <c r="M35" s="336"/>
-      <c r="N35" s="336"/>
-      <c r="O35" s="336"/>
-      <c r="P35" s="336"/>
-      <c r="Q35" s="336"/>
-      <c r="R35" s="336"/>
-      <c r="S35" s="336"/>
-      <c r="T35" s="336"/>
-      <c r="U35" s="336"/>
-      <c r="V35" s="336"/>
-      <c r="W35" s="336"/>
-      <c r="X35" s="337"/>
+      <c r="B35" s="194"/>
+      <c r="C35" s="194"/>
+      <c r="D35" s="194"/>
+      <c r="E35" s="194"/>
+      <c r="F35" s="194"/>
+      <c r="G35" s="194"/>
+      <c r="H35" s="194"/>
+      <c r="I35" s="194"/>
+      <c r="J35" s="194"/>
+      <c r="K35" s="194"/>
+      <c r="L35" s="194"/>
+      <c r="M35" s="194"/>
+      <c r="N35" s="194"/>
+      <c r="O35" s="194"/>
+      <c r="P35" s="194"/>
+      <c r="Q35" s="194"/>
+      <c r="R35" s="194"/>
+      <c r="S35" s="194"/>
+      <c r="T35" s="194"/>
+      <c r="U35" s="194"/>
+      <c r="V35" s="194"/>
+      <c r="W35" s="194"/>
+      <c r="X35" s="195"/>
     </row>
   </sheetData>
-  <mergeCells count="29">
-    <mergeCell ref="U23:W23"/>
-    <mergeCell ref="R3:X4"/>
-    <mergeCell ref="R5:X6"/>
-    <mergeCell ref="U14:W14"/>
-    <mergeCell ref="U15:W15"/>
-    <mergeCell ref="U11:W11"/>
-    <mergeCell ref="U12:W12"/>
+  <mergeCells count="30">
     <mergeCell ref="A1:X1"/>
     <mergeCell ref="U33:W33"/>
     <mergeCell ref="U16:W16"/>
@@ -17089,12 +16962,20 @@
     <mergeCell ref="U20:W20"/>
     <mergeCell ref="U21:W21"/>
     <mergeCell ref="U22:W22"/>
+    <mergeCell ref="R2:X2"/>
     <mergeCell ref="U34:W34"/>
     <mergeCell ref="A35:X35"/>
     <mergeCell ref="U28:W28"/>
     <mergeCell ref="U29:W29"/>
     <mergeCell ref="U30:W30"/>
     <mergeCell ref="U31:W31"/>
+    <mergeCell ref="U23:W23"/>
+    <mergeCell ref="R3:X4"/>
+    <mergeCell ref="R5:X6"/>
+    <mergeCell ref="U14:W14"/>
+    <mergeCell ref="U15:W15"/>
+    <mergeCell ref="U11:W11"/>
+    <mergeCell ref="U12:W12"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.47244094488188981" right="0.31496062992125984" top="0.55118110236220474" bottom="0.74803149606299213" header="0.51181102362204722" footer="0.51181102362204722"/>

</xml_diff>

<commit_message>
Fix: Resolve welder ID duplication, add date filtering for result sync, and force ascending DWG sort on extraction
</commit_message>
<xml_diff>
--- a/Na-aba/home/data/SISGI-KOGAS-RT-001.xlsx
+++ b/Na-aba/home/data/SISGI-KOGAS-RT-001.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jjch2\Desktop\보고서\Project PROVIDENCE\Request\PMI\Na-aba\home\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{500826BB-A592-4F9E-BFA2-87180EEC48F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C2BDC90-995D-404C-BCA5-2C215867BDDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EBDC5234-EA45-45C7-9BE3-C0C611B2FCE5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{EBDC5234-EA45-45C7-9BE3-C0C611B2FCE5}"/>
   </bookViews>
   <sheets>
     <sheet name="RT(갑) 1" sheetId="10" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="232">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="231">
   <si>
     <t>□</t>
   </si>
@@ -921,10 +921,6 @@
   </si>
   <si>
     <t>■  Fe                 □  Al</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>KGW-TL-00</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
@@ -2284,18 +2280,459 @@
     <xf numFmtId="176" fontId="15" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="8" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="8" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="8" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="44" xfId="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="6" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="45" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="44" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="42" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="43" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="42" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="179" fontId="8" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="8" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="8" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="178" fontId="8" fillId="0" borderId="39" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="178" fontId="8" fillId="0" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="178" fontId="8" fillId="0" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
@@ -2305,27 +2742,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="45" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2360,426 +2776,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="179" fontId="8" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="8" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="8" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="178" fontId="8" fillId="0" borderId="39" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="178" fontId="8" fillId="0" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="178" fontId="8" fillId="0" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="42" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="43" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="42" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="45" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="44" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="6" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="44" xfId="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="8" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="8" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="8" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -14531,44 +14527,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="21.75" customHeight="1">
-      <c r="A1" s="199" t="s">
+      <c r="A1" s="201" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="273"/>
-      <c r="C1" s="273"/>
-      <c r="D1" s="273"/>
-      <c r="E1" s="273"/>
-      <c r="F1" s="273"/>
-      <c r="G1" s="273"/>
-      <c r="H1" s="273"/>
-      <c r="I1" s="273"/>
-      <c r="J1" s="273"/>
-      <c r="K1" s="273"/>
-      <c r="L1" s="273"/>
-      <c r="M1" s="273"/>
-      <c r="N1" s="273"/>
-      <c r="O1" s="273"/>
-      <c r="P1" s="273"/>
+      <c r="B1" s="202"/>
+      <c r="C1" s="202"/>
+      <c r="D1" s="202"/>
+      <c r="E1" s="202"/>
+      <c r="F1" s="202"/>
+      <c r="G1" s="202"/>
+      <c r="H1" s="202"/>
+      <c r="I1" s="202"/>
+      <c r="J1" s="202"/>
+      <c r="K1" s="202"/>
+      <c r="L1" s="202"/>
+      <c r="M1" s="202"/>
+      <c r="N1" s="202"/>
+      <c r="O1" s="202"/>
+      <c r="P1" s="202"/>
     </row>
     <row r="2" spans="1:16" ht="18.75" customHeight="1">
-      <c r="A2" s="199" t="s">
+      <c r="A2" s="201" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="273"/>
-      <c r="C2" s="273"/>
-      <c r="D2" s="273"/>
-      <c r="E2" s="273"/>
-      <c r="F2" s="273"/>
-      <c r="G2" s="273"/>
-      <c r="H2" s="273"/>
-      <c r="I2" s="273"/>
-      <c r="J2" s="273"/>
-      <c r="K2" s="273"/>
-      <c r="L2" s="273"/>
-      <c r="M2" s="273"/>
-      <c r="N2" s="273"/>
-      <c r="O2" s="273"/>
-      <c r="P2" s="273"/>
+      <c r="B2" s="202"/>
+      <c r="C2" s="202"/>
+      <c r="D2" s="202"/>
+      <c r="E2" s="202"/>
+      <c r="F2" s="202"/>
+      <c r="G2" s="202"/>
+      <c r="H2" s="202"/>
+      <c r="I2" s="202"/>
+      <c r="J2" s="202"/>
+      <c r="K2" s="202"/>
+      <c r="L2" s="202"/>
+      <c r="M2" s="202"/>
+      <c r="N2" s="202"/>
+      <c r="O2" s="202"/>
+      <c r="P2" s="202"/>
     </row>
     <row r="3" spans="1:16" ht="12" customHeight="1">
       <c r="A3" s="3"/>
@@ -14584,152 +14580,152 @@
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
-      <c r="N3" s="274"/>
-      <c r="O3" s="275"/>
-      <c r="P3" s="275"/>
+      <c r="N3" s="268"/>
+      <c r="O3" s="234"/>
+      <c r="P3" s="234"/>
     </row>
     <row r="4" spans="1:16" ht="15.75" customHeight="1">
       <c r="A4" s="5"/>
       <c r="B4" s="6"/>
-      <c r="C4" s="276" t="s">
+      <c r="C4" s="269" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="277"/>
-      <c r="E4" s="277"/>
-      <c r="F4" s="277"/>
-      <c r="G4" s="277"/>
-      <c r="H4" s="277"/>
-      <c r="I4" s="277"/>
-      <c r="J4" s="277"/>
-      <c r="K4" s="278"/>
-      <c r="L4" s="228" t="s">
+      <c r="D4" s="270"/>
+      <c r="E4" s="270"/>
+      <c r="F4" s="270"/>
+      <c r="G4" s="270"/>
+      <c r="H4" s="270"/>
+      <c r="I4" s="270"/>
+      <c r="J4" s="270"/>
+      <c r="K4" s="271"/>
+      <c r="L4" s="286" t="s">
         <v>4</v>
       </c>
-      <c r="M4" s="229"/>
-      <c r="N4" s="285" t="s">
+      <c r="M4" s="287"/>
+      <c r="N4" s="278" t="s">
         <v>169</v>
       </c>
-      <c r="O4" s="286"/>
-      <c r="P4" s="287"/>
+      <c r="O4" s="279"/>
+      <c r="P4" s="280"/>
     </row>
     <row r="5" spans="1:16" ht="12.75" customHeight="1">
       <c r="A5" s="5"/>
       <c r="B5" s="6"/>
-      <c r="C5" s="279" t="s">
+      <c r="C5" s="272" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="279"/>
-      <c r="E5" s="279"/>
-      <c r="F5" s="279"/>
-      <c r="G5" s="279"/>
-      <c r="H5" s="279"/>
-      <c r="I5" s="279"/>
-      <c r="J5" s="279"/>
-      <c r="K5" s="280"/>
-      <c r="L5" s="230" t="s">
+      <c r="D5" s="272"/>
+      <c r="E5" s="272"/>
+      <c r="F5" s="272"/>
+      <c r="G5" s="272"/>
+      <c r="H5" s="272"/>
+      <c r="I5" s="272"/>
+      <c r="J5" s="272"/>
+      <c r="K5" s="273"/>
+      <c r="L5" s="288" t="s">
         <v>6</v>
       </c>
-      <c r="M5" s="231"/>
-      <c r="N5" s="288"/>
-      <c r="O5" s="289"/>
-      <c r="P5" s="290"/>
+      <c r="M5" s="289"/>
+      <c r="N5" s="281"/>
+      <c r="O5" s="282"/>
+      <c r="P5" s="283"/>
     </row>
     <row r="6" spans="1:16" ht="12.75" customHeight="1">
       <c r="A6" s="5"/>
       <c r="B6" s="6"/>
-      <c r="C6" s="281" t="s">
+      <c r="C6" s="274" t="s">
         <v>168</v>
       </c>
-      <c r="D6" s="281"/>
-      <c r="E6" s="281"/>
-      <c r="F6" s="281"/>
-      <c r="G6" s="281"/>
-      <c r="H6" s="281"/>
-      <c r="I6" s="281"/>
-      <c r="J6" s="281"/>
-      <c r="K6" s="282"/>
-      <c r="L6" s="232" t="s">
+      <c r="D6" s="274"/>
+      <c r="E6" s="274"/>
+      <c r="F6" s="274"/>
+      <c r="G6" s="274"/>
+      <c r="H6" s="274"/>
+      <c r="I6" s="274"/>
+      <c r="J6" s="274"/>
+      <c r="K6" s="275"/>
+      <c r="L6" s="290" t="s">
         <v>7</v>
       </c>
-      <c r="M6" s="233"/>
-      <c r="N6" s="242" t="s">
+      <c r="M6" s="291"/>
+      <c r="N6" s="300" t="s">
         <v>170</v>
       </c>
-      <c r="O6" s="252"/>
-      <c r="P6" s="253"/>
+      <c r="O6" s="310"/>
+      <c r="P6" s="311"/>
     </row>
     <row r="7" spans="1:16" ht="12.75" customHeight="1">
       <c r="A7" s="7"/>
       <c r="B7" s="8"/>
-      <c r="C7" s="283" t="s">
+      <c r="C7" s="276" t="s">
         <v>8</v>
       </c>
-      <c r="D7" s="283"/>
-      <c r="E7" s="283"/>
-      <c r="F7" s="283"/>
-      <c r="G7" s="283"/>
-      <c r="H7" s="283"/>
-      <c r="I7" s="283"/>
-      <c r="J7" s="283"/>
-      <c r="K7" s="284"/>
-      <c r="L7" s="234" t="s">
+      <c r="D7" s="276"/>
+      <c r="E7" s="276"/>
+      <c r="F7" s="276"/>
+      <c r="G7" s="276"/>
+      <c r="H7" s="276"/>
+      <c r="I7" s="276"/>
+      <c r="J7" s="276"/>
+      <c r="K7" s="277"/>
+      <c r="L7" s="292" t="s">
         <v>9</v>
       </c>
-      <c r="M7" s="235"/>
-      <c r="N7" s="254"/>
-      <c r="O7" s="255"/>
-      <c r="P7" s="256"/>
+      <c r="M7" s="293"/>
+      <c r="N7" s="312"/>
+      <c r="O7" s="313"/>
+      <c r="P7" s="314"/>
     </row>
     <row r="8" spans="1:16" s="12" customFormat="1" ht="24" customHeight="1">
       <c r="A8" s="9"/>
       <c r="B8" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="236" t="s">
-        <v>230</v>
-      </c>
-      <c r="D8" s="237"/>
-      <c r="E8" s="237"/>
-      <c r="F8" s="237"/>
-      <c r="G8" s="237"/>
-      <c r="H8" s="237"/>
-      <c r="I8" s="238"/>
+      <c r="C8" s="294" t="s">
+        <v>229</v>
+      </c>
+      <c r="D8" s="295"/>
+      <c r="E8" s="295"/>
+      <c r="F8" s="295"/>
+      <c r="G8" s="295"/>
+      <c r="H8" s="295"/>
+      <c r="I8" s="296"/>
       <c r="J8" s="11"/>
       <c r="K8" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="L8" s="239" t="s">
+      <c r="L8" s="297" t="s">
         <v>206</v>
       </c>
-      <c r="M8" s="240"/>
-      <c r="N8" s="240"/>
-      <c r="O8" s="240"/>
-      <c r="P8" s="241"/>
+      <c r="M8" s="298"/>
+      <c r="N8" s="298"/>
+      <c r="O8" s="298"/>
+      <c r="P8" s="299"/>
     </row>
     <row r="9" spans="1:16" s="12" customFormat="1" ht="13.5" customHeight="1">
       <c r="A9" s="13"/>
       <c r="B9" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="242" t="s">
+      <c r="C9" s="300" t="s">
         <v>205</v>
       </c>
-      <c r="D9" s="243"/>
-      <c r="E9" s="243"/>
-      <c r="F9" s="243"/>
-      <c r="G9" s="243"/>
-      <c r="H9" s="243"/>
-      <c r="I9" s="244"/>
+      <c r="D9" s="301"/>
+      <c r="E9" s="301"/>
+      <c r="F9" s="301"/>
+      <c r="G9" s="301"/>
+      <c r="H9" s="301"/>
+      <c r="I9" s="302"/>
       <c r="J9" s="15"/>
       <c r="K9" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="L9" s="259" t="s">
+      <c r="L9" s="316" t="s">
         <v>217</v>
       </c>
-      <c r="M9" s="260"/>
-      <c r="N9" s="260"/>
-      <c r="O9" s="260"/>
+      <c r="M9" s="317"/>
+      <c r="N9" s="317"/>
+      <c r="O9" s="317"/>
       <c r="P9" s="116" t="s">
         <v>14</v>
       </c>
@@ -14739,21 +14735,21 @@
       <c r="B10" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="245"/>
-      <c r="D10" s="246"/>
-      <c r="E10" s="246"/>
-      <c r="F10" s="246"/>
-      <c r="G10" s="246"/>
-      <c r="H10" s="246"/>
-      <c r="I10" s="247"/>
+      <c r="C10" s="303"/>
+      <c r="D10" s="304"/>
+      <c r="E10" s="304"/>
+      <c r="F10" s="304"/>
+      <c r="G10" s="304"/>
+      <c r="H10" s="304"/>
+      <c r="I10" s="305"/>
       <c r="J10" s="18"/>
       <c r="K10" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="L10" s="261"/>
-      <c r="M10" s="262"/>
-      <c r="N10" s="262"/>
-      <c r="O10" s="262"/>
+      <c r="L10" s="318"/>
+      <c r="M10" s="319"/>
+      <c r="N10" s="319"/>
+      <c r="O10" s="319"/>
       <c r="P10" s="117" t="s">
         <v>171</v>
       </c>
@@ -14786,13 +14782,13 @@
       <c r="K11" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="L11" s="221" t="s">
+      <c r="L11" s="261" t="s">
         <v>177</v>
       </c>
-      <c r="M11" s="222"/>
-      <c r="N11" s="222"/>
-      <c r="O11" s="222"/>
-      <c r="P11" s="267"/>
+      <c r="M11" s="262"/>
+      <c r="N11" s="262"/>
+      <c r="O11" s="262"/>
+      <c r="P11" s="263"/>
     </row>
     <row r="12" spans="1:16" s="12" customFormat="1" ht="13.5" customHeight="1">
       <c r="A12" s="21"/>
@@ -14814,13 +14810,13 @@
       <c r="I12" s="123"/>
       <c r="J12" s="24"/>
       <c r="K12" s="22" t="s">
-        <v>224</v>
-      </c>
-      <c r="L12" s="268"/>
-      <c r="M12" s="269"/>
-      <c r="N12" s="269"/>
-      <c r="O12" s="269"/>
-      <c r="P12" s="270"/>
+        <v>223</v>
+      </c>
+      <c r="L12" s="264"/>
+      <c r="M12" s="265"/>
+      <c r="N12" s="265"/>
+      <c r="O12" s="265"/>
+      <c r="P12" s="266"/>
     </row>
     <row r="13" spans="1:16" s="12" customFormat="1" ht="13.5" customHeight="1">
       <c r="A13" s="19"/>
@@ -14853,10 +14849,10 @@
       <c r="L13" s="137" t="s">
         <v>32</v>
       </c>
-      <c r="M13" s="265">
+      <c r="M13" s="320">
         <v>15.9</v>
       </c>
-      <c r="N13" s="265"/>
+      <c r="N13" s="320"/>
       <c r="O13" s="119" t="s">
         <v>18</v>
       </c>
@@ -14889,8 +14885,8 @@
       <c r="L14" s="140" t="s">
         <v>39</v>
       </c>
-      <c r="M14" s="266"/>
-      <c r="N14" s="266"/>
+      <c r="M14" s="221"/>
+      <c r="N14" s="221"/>
       <c r="O14" s="122" t="s">
         <v>173</v>
       </c>
@@ -14906,18 +14902,18 @@
       <c r="C15" s="118" t="s">
         <v>172</v>
       </c>
-      <c r="D15" s="257" t="s">
+      <c r="D15" s="210" t="s">
         <v>42</v>
       </c>
-      <c r="E15" s="258"/>
-      <c r="F15" s="258"/>
+      <c r="E15" s="315"/>
+      <c r="F15" s="315"/>
       <c r="G15" s="119" t="s">
         <v>164</v>
       </c>
-      <c r="H15" s="257" t="s">
+      <c r="H15" s="210" t="s">
         <v>43</v>
       </c>
-      <c r="I15" s="329"/>
+      <c r="I15" s="211"/>
       <c r="J15" s="15"/>
       <c r="K15" s="14" t="s">
         <v>44</v>
@@ -14925,10 +14921,10 @@
       <c r="L15" s="143" t="s">
         <v>207</v>
       </c>
-      <c r="M15" s="263">
+      <c r="M15" s="222">
         <v>2</v>
       </c>
-      <c r="N15" s="263"/>
+      <c r="N15" s="222"/>
       <c r="O15" s="119" t="s">
         <v>18</v>
       </c>
@@ -14944,18 +14940,18 @@
       <c r="C16" s="121" t="s">
         <v>172</v>
       </c>
-      <c r="D16" s="271" t="s">
+      <c r="D16" s="242" t="s">
         <v>46</v>
       </c>
-      <c r="E16" s="272"/>
-      <c r="F16" s="272"/>
+      <c r="E16" s="267"/>
+      <c r="F16" s="267"/>
       <c r="G16" s="122" t="s">
         <v>18</v>
       </c>
-      <c r="H16" s="271" t="s">
+      <c r="H16" s="242" t="s">
         <v>47</v>
       </c>
-      <c r="I16" s="298"/>
+      <c r="I16" s="243"/>
       <c r="J16" s="24"/>
       <c r="K16" s="22" t="s">
         <v>48</v>
@@ -14963,8 +14959,8 @@
       <c r="L16" s="131" t="s">
         <v>49</v>
       </c>
-      <c r="M16" s="264"/>
-      <c r="N16" s="264"/>
+      <c r="M16" s="224"/>
+      <c r="N16" s="224"/>
       <c r="O16" s="122" t="s">
         <v>173</v>
       </c>
@@ -14996,13 +14992,13 @@
       <c r="K17" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="L17" s="332" t="s">
+      <c r="L17" s="197" t="s">
         <v>178</v>
       </c>
-      <c r="M17" s="333"/>
-      <c r="N17" s="333"/>
-      <c r="O17" s="333"/>
-      <c r="P17" s="334"/>
+      <c r="M17" s="214"/>
+      <c r="N17" s="214"/>
+      <c r="O17" s="214"/>
+      <c r="P17" s="215"/>
     </row>
     <row r="18" spans="1:16" s="12" customFormat="1" ht="12.75" customHeight="1">
       <c r="A18" s="13"/>
@@ -15021,37 +15017,37 @@
       </c>
       <c r="G18" s="135"/>
       <c r="H18" s="132" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="I18" s="136"/>
       <c r="J18" s="18"/>
       <c r="K18" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="L18" s="335" t="s">
+      <c r="L18" s="198" t="s">
         <v>179</v>
       </c>
-      <c r="M18" s="336"/>
-      <c r="N18" s="336"/>
-      <c r="O18" s="336"/>
-      <c r="P18" s="337"/>
+      <c r="M18" s="216"/>
+      <c r="N18" s="216"/>
+      <c r="O18" s="216"/>
+      <c r="P18" s="217"/>
     </row>
     <row r="19" spans="1:16" s="31" customFormat="1" ht="13.5" customHeight="1">
       <c r="A19" s="28"/>
       <c r="B19" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="C19" s="327" t="s">
+      <c r="C19" s="208" t="s">
         <v>56</v>
       </c>
-      <c r="D19" s="349" t="s">
+      <c r="D19" s="193" t="s">
+        <v>227</v>
+      </c>
+      <c r="E19" s="195" t="s">
+        <v>226</v>
+      </c>
+      <c r="F19" s="191" t="s">
         <v>228</v>
-      </c>
-      <c r="E19" s="351" t="s">
-        <v>227</v>
-      </c>
-      <c r="F19" s="347" t="s">
-        <v>229</v>
       </c>
       <c r="G19" s="20" t="s">
         <v>18</v>
@@ -15081,10 +15077,10 @@
       <c r="B20" s="22" t="s">
         <v>60</v>
       </c>
-      <c r="C20" s="328"/>
-      <c r="D20" s="350"/>
-      <c r="E20" s="352"/>
-      <c r="F20" s="348"/>
+      <c r="C20" s="209"/>
+      <c r="D20" s="194"/>
+      <c r="E20" s="196"/>
+      <c r="F20" s="192"/>
       <c r="G20" s="23" t="s">
         <v>173</v>
       </c>
@@ -15096,11 +15092,11 @@
       <c r="K20" s="22" t="s">
         <v>62</v>
       </c>
-      <c r="L20" s="340" t="s">
+      <c r="L20" s="220" t="s">
         <v>181</v>
       </c>
-      <c r="M20" s="266"/>
-      <c r="N20" s="266"/>
+      <c r="M20" s="221"/>
+      <c r="N20" s="221"/>
       <c r="O20" s="122" t="s">
         <v>164</v>
       </c>
@@ -15113,15 +15109,15 @@
       <c r="B21" s="114" t="s">
         <v>166</v>
       </c>
-      <c r="C21" s="303" t="s">
+      <c r="C21" s="246" t="s">
         <v>167</v>
       </c>
-      <c r="D21" s="304"/>
-      <c r="E21" s="304"/>
-      <c r="F21" s="304"/>
-      <c r="G21" s="304"/>
-      <c r="H21" s="304"/>
-      <c r="I21" s="330"/>
+      <c r="D21" s="247"/>
+      <c r="E21" s="247"/>
+      <c r="F21" s="247"/>
+      <c r="G21" s="247"/>
+      <c r="H21" s="247"/>
+      <c r="I21" s="212"/>
       <c r="J21" s="30"/>
       <c r="K21" s="14" t="s">
         <v>213</v>
@@ -15145,15 +15141,15 @@
       <c r="B22" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="C22" s="305" t="s">
-        <v>226</v>
-      </c>
-      <c r="D22" s="306"/>
-      <c r="E22" s="306"/>
-      <c r="F22" s="306"/>
-      <c r="G22" s="306"/>
-      <c r="H22" s="306"/>
-      <c r="I22" s="331"/>
+      <c r="C22" s="248" t="s">
+        <v>225</v>
+      </c>
+      <c r="D22" s="249"/>
+      <c r="E22" s="249"/>
+      <c r="F22" s="249"/>
+      <c r="G22" s="249"/>
+      <c r="H22" s="249"/>
+      <c r="I22" s="213"/>
       <c r="J22" s="34"/>
       <c r="K22" s="22" t="s">
         <v>214</v>
@@ -15181,10 +15177,10 @@
       <c r="D23" s="145" t="s">
         <v>187</v>
       </c>
-      <c r="E23" s="353">
+      <c r="E23" s="199">
         <v>375</v>
       </c>
-      <c r="F23" s="354"/>
+      <c r="F23" s="200"/>
       <c r="G23" s="119" t="s">
         <v>18</v>
       </c>
@@ -15196,15 +15192,15 @@
       <c r="K23" s="14" t="s">
         <v>203</v>
       </c>
-      <c r="L23" s="311" t="s">
+      <c r="L23" s="254" t="s">
         <v>210</v>
       </c>
-      <c r="M23" s="312"/>
-      <c r="N23" s="312"/>
-      <c r="O23" s="309" t="s">
+      <c r="M23" s="255"/>
+      <c r="N23" s="255"/>
+      <c r="O23" s="252" t="s">
         <v>211</v>
       </c>
-      <c r="P23" s="310"/>
+      <c r="P23" s="253"/>
     </row>
     <row r="24" spans="1:16" s="31" customFormat="1" ht="23.1" customHeight="1">
       <c r="A24" s="113"/>
@@ -15215,10 +15211,10 @@
       <c r="D24" s="145" t="s">
         <v>189</v>
       </c>
-      <c r="E24" s="299">
+      <c r="E24" s="244">
         <v>17.899999999999999</v>
       </c>
-      <c r="F24" s="300"/>
+      <c r="F24" s="245"/>
       <c r="G24" s="125" t="s">
         <v>173</v>
       </c>
@@ -15230,15 +15226,15 @@
       <c r="K24" s="176" t="s">
         <v>204</v>
       </c>
-      <c r="L24" s="311" t="s">
+      <c r="L24" s="254" t="s">
         <v>220</v>
       </c>
-      <c r="M24" s="312"/>
-      <c r="N24" s="312"/>
-      <c r="O24" s="307" t="s">
+      <c r="M24" s="255"/>
+      <c r="N24" s="255"/>
+      <c r="O24" s="250" t="s">
         <v>221</v>
       </c>
-      <c r="P24" s="308"/>
+      <c r="P24" s="251"/>
     </row>
     <row r="25" spans="1:16" s="31" customFormat="1" ht="13.5" customHeight="1">
       <c r="A25" s="28"/>
@@ -15246,11 +15242,11 @@
         <v>64</v>
       </c>
       <c r="C25" s="118"/>
-      <c r="D25" s="345" t="s">
+      <c r="D25" s="189" t="s">
         <v>209</v>
       </c>
-      <c r="E25" s="346"/>
-      <c r="F25" s="346"/>
+      <c r="E25" s="190"/>
+      <c r="F25" s="190"/>
       <c r="G25" s="119" t="s">
         <v>173</v>
       </c>
@@ -15265,12 +15261,12 @@
       <c r="L25" s="143" t="s">
         <v>66</v>
       </c>
-      <c r="M25" s="263" t="s">
+      <c r="M25" s="222" t="s">
         <v>182</v>
       </c>
-      <c r="N25" s="263"/>
-      <c r="O25" s="263"/>
-      <c r="P25" s="341"/>
+      <c r="N25" s="222"/>
+      <c r="O25" s="222"/>
+      <c r="P25" s="223"/>
     </row>
     <row r="26" spans="1:16" s="31" customFormat="1" ht="13.5" customHeight="1">
       <c r="A26" s="35"/>
@@ -15301,24 +15297,24 @@
       <c r="L26" s="124" t="s">
         <v>69</v>
       </c>
-      <c r="M26" s="264" t="s">
+      <c r="M26" s="224" t="s">
         <v>183</v>
       </c>
-      <c r="N26" s="264"/>
-      <c r="O26" s="264"/>
-      <c r="P26" s="342"/>
+      <c r="N26" s="224"/>
+      <c r="O26" s="224"/>
+      <c r="P26" s="225"/>
     </row>
     <row r="27" spans="1:16" s="31" customFormat="1" ht="13.5" customHeight="1">
       <c r="A27" s="28"/>
       <c r="B27" s="151" t="s">
         <v>70</v>
       </c>
-      <c r="C27" s="332"/>
-      <c r="D27" s="343" t="s">
+      <c r="C27" s="197"/>
+      <c r="D27" s="226" t="s">
         <v>191</v>
       </c>
-      <c r="E27" s="333"/>
-      <c r="F27" s="333" t="s">
+      <c r="E27" s="214"/>
+      <c r="F27" s="214" t="s">
         <v>192</v>
       </c>
       <c r="G27" s="119" t="s">
@@ -15353,10 +15349,10 @@
       <c r="B28" s="152" t="s">
         <v>75</v>
       </c>
-      <c r="C28" s="335"/>
-      <c r="D28" s="344"/>
-      <c r="E28" s="336"/>
-      <c r="F28" s="336"/>
+      <c r="C28" s="198"/>
+      <c r="D28" s="227"/>
+      <c r="E28" s="216"/>
+      <c r="F28" s="216"/>
       <c r="G28" s="122" t="s">
         <v>18</v>
       </c>
@@ -15383,38 +15379,38 @@
       <c r="B29" s="154" t="s">
         <v>79</v>
       </c>
-      <c r="C29" s="313" t="s">
+      <c r="C29" s="256" t="s">
         <v>193</v>
       </c>
-      <c r="D29" s="314"/>
-      <c r="E29" s="315"/>
-      <c r="F29" s="315"/>
-      <c r="G29" s="315"/>
-      <c r="H29" s="316"/>
-      <c r="I29" s="317"/>
+      <c r="D29" s="257"/>
+      <c r="E29" s="258"/>
+      <c r="F29" s="258"/>
+      <c r="G29" s="258"/>
+      <c r="H29" s="259"/>
+      <c r="I29" s="260"/>
       <c r="J29" s="40"/>
       <c r="K29" s="41" t="s">
         <v>80</v>
       </c>
-      <c r="L29" s="223">
+      <c r="L29" s="327">
         <v>0.32</v>
       </c>
-      <c r="M29" s="224"/>
-      <c r="N29" s="224"/>
-      <c r="O29" s="224"/>
-      <c r="P29" s="225"/>
+      <c r="M29" s="328"/>
+      <c r="N29" s="328"/>
+      <c r="O29" s="328"/>
+      <c r="P29" s="329"/>
     </row>
     <row r="30" spans="1:16" s="31" customFormat="1" ht="12.75" customHeight="1">
       <c r="A30" s="28"/>
       <c r="B30" s="119" t="s">
         <v>81</v>
       </c>
-      <c r="C30" s="248" t="s">
+      <c r="C30" s="306" t="s">
         <v>200</v>
       </c>
-      <c r="D30" s="249"/>
-      <c r="E30" s="249"/>
-      <c r="F30" s="249"/>
+      <c r="D30" s="307"/>
+      <c r="E30" s="307"/>
+      <c r="F30" s="307"/>
       <c r="G30" s="119" t="s">
         <v>164</v>
       </c>
@@ -15426,12 +15422,12 @@
       <c r="K30" s="14" t="s">
         <v>83</v>
       </c>
-      <c r="L30" s="221" t="s">
+      <c r="L30" s="261" t="s">
         <v>202</v>
       </c>
-      <c r="M30" s="222"/>
-      <c r="N30" s="222"/>
-      <c r="O30" s="222"/>
+      <c r="M30" s="262"/>
+      <c r="N30" s="262"/>
+      <c r="O30" s="262"/>
       <c r="P30" s="175" t="s">
         <v>184</v>
       </c>
@@ -15441,10 +15437,10 @@
       <c r="B31" s="156" t="s">
         <v>84</v>
       </c>
-      <c r="C31" s="250"/>
-      <c r="D31" s="251"/>
-      <c r="E31" s="251"/>
-      <c r="F31" s="251"/>
+      <c r="C31" s="308"/>
+      <c r="D31" s="309"/>
+      <c r="E31" s="309"/>
+      <c r="F31" s="309"/>
       <c r="G31" s="43" t="s">
         <v>194</v>
       </c>
@@ -15456,17 +15452,17 @@
       <c r="K31" s="43" t="s">
         <v>86</v>
       </c>
-      <c r="L31" s="218" t="s">
+      <c r="L31" s="324" t="s">
         <v>185</v>
       </c>
-      <c r="M31" s="219"/>
-      <c r="N31" s="219"/>
-      <c r="O31" s="219"/>
-      <c r="P31" s="220"/>
+      <c r="M31" s="325"/>
+      <c r="N31" s="325"/>
+      <c r="O31" s="325"/>
+      <c r="P31" s="326"/>
     </row>
     <row r="32" spans="1:16" s="31" customFormat="1" ht="6.75" customHeight="1">
       <c r="A32" s="35"/>
-      <c r="B32" s="226" t="s">
+      <c r="B32" s="284" t="s">
         <v>87</v>
       </c>
       <c r="C32" s="45"/>
@@ -15486,7 +15482,7 @@
     </row>
     <row r="33" spans="1:16" s="31" customFormat="1" ht="13.5" customHeight="1">
       <c r="A33" s="35"/>
-      <c r="B33" s="227"/>
+      <c r="B33" s="285"/>
       <c r="C33" s="25" t="s">
         <v>165</v>
       </c>
@@ -15681,117 +15677,117 @@
       <c r="B43" s="51" t="s">
         <v>88</v>
       </c>
-      <c r="C43" s="323"/>
-      <c r="D43" s="323"/>
-      <c r="E43" s="323"/>
-      <c r="F43" s="338" t="s">
+      <c r="C43" s="204"/>
+      <c r="D43" s="204"/>
+      <c r="E43" s="204"/>
+      <c r="F43" s="218" t="s">
         <v>89</v>
       </c>
-      <c r="G43" s="339"/>
+      <c r="G43" s="219"/>
       <c r="H43" s="159"/>
       <c r="I43" s="52"/>
       <c r="J43" s="53"/>
-      <c r="K43" s="324" t="s">
+      <c r="K43" s="205" t="s">
         <v>197</v>
       </c>
-      <c r="L43" s="325"/>
-      <c r="M43" s="325"/>
-      <c r="N43" s="325"/>
-      <c r="O43" s="325"/>
-      <c r="P43" s="326"/>
+      <c r="L43" s="206"/>
+      <c r="M43" s="206"/>
+      <c r="N43" s="206"/>
+      <c r="O43" s="206"/>
+      <c r="P43" s="207"/>
     </row>
     <row r="44" spans="1:16" ht="15.75" customHeight="1">
       <c r="A44" s="55"/>
       <c r="B44" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="C44" s="294" t="s">
+      <c r="C44" s="203" t="s">
         <v>195</v>
       </c>
-      <c r="D44" s="294"/>
-      <c r="E44" s="294"/>
-      <c r="F44" s="301" t="s">
+      <c r="D44" s="203"/>
+      <c r="E44" s="203"/>
+      <c r="F44" s="231" t="s">
         <v>91</v>
       </c>
-      <c r="G44" s="302"/>
+      <c r="G44" s="232"/>
       <c r="H44" s="126" t="s">
         <v>196</v>
       </c>
-      <c r="K44" s="215">
+      <c r="K44" s="321">
         <v>45821</v>
       </c>
-      <c r="L44" s="215"/>
+      <c r="L44" s="321"/>
       <c r="M44" s="180" t="s">
-        <v>223</v>
-      </c>
-      <c r="N44" s="216">
+        <v>222</v>
+      </c>
+      <c r="N44" s="322">
         <v>45827</v>
       </c>
-      <c r="O44" s="216"/>
-      <c r="P44" s="217"/>
+      <c r="O44" s="322"/>
+      <c r="P44" s="323"/>
     </row>
     <row r="45" spans="1:16" ht="12.75" customHeight="1">
       <c r="A45" s="55"/>
       <c r="B45" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C45" s="294"/>
-      <c r="D45" s="294"/>
-      <c r="E45" s="294"/>
-      <c r="F45" s="301" t="s">
+      <c r="C45" s="203"/>
+      <c r="D45" s="203"/>
+      <c r="E45" s="203"/>
+      <c r="F45" s="231" t="s">
         <v>89</v>
       </c>
-      <c r="G45" s="302"/>
+      <c r="G45" s="232"/>
       <c r="H45" s="126"/>
       <c r="I45" s="49"/>
       <c r="J45" s="15"/>
-      <c r="K45" s="291" t="s">
+      <c r="K45" s="236" t="s">
         <v>93</v>
       </c>
-      <c r="L45" s="292"/>
-      <c r="M45" s="292"/>
-      <c r="N45" s="292"/>
-      <c r="O45" s="292"/>
-      <c r="P45" s="293"/>
+      <c r="L45" s="237"/>
+      <c r="M45" s="237"/>
+      <c r="N45" s="237"/>
+      <c r="O45" s="237"/>
+      <c r="P45" s="238"/>
     </row>
     <row r="46" spans="1:16" ht="15" customHeight="1">
       <c r="A46" s="55"/>
       <c r="B46" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="C46" s="294" t="s">
+      <c r="C46" s="203" t="s">
         <v>208</v>
       </c>
-      <c r="D46" s="294"/>
-      <c r="E46" s="294"/>
-      <c r="F46" s="301" t="s">
+      <c r="D46" s="203"/>
+      <c r="E46" s="203"/>
+      <c r="F46" s="231" t="s">
         <v>91</v>
       </c>
-      <c r="G46" s="302"/>
+      <c r="G46" s="232"/>
       <c r="H46" s="126" t="s">
         <v>212</v>
       </c>
       <c r="I46" s="49"/>
       <c r="J46" s="24"/>
-      <c r="K46" s="295"/>
-      <c r="L46" s="296"/>
-      <c r="M46" s="296"/>
-      <c r="N46" s="296"/>
-      <c r="O46" s="296"/>
-      <c r="P46" s="297"/>
+      <c r="K46" s="239"/>
+      <c r="L46" s="240"/>
+      <c r="M46" s="240"/>
+      <c r="N46" s="240"/>
+      <c r="O46" s="240"/>
+      <c r="P46" s="241"/>
     </row>
     <row r="47" spans="1:16" ht="13.5" customHeight="1">
       <c r="A47" s="55"/>
       <c r="B47" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="C47" s="294"/>
-      <c r="D47" s="294"/>
-      <c r="E47" s="294"/>
-      <c r="F47" s="301" t="s">
+      <c r="C47" s="203"/>
+      <c r="D47" s="203"/>
+      <c r="E47" s="203"/>
+      <c r="F47" s="231" t="s">
         <v>89</v>
       </c>
-      <c r="G47" s="302"/>
+      <c r="G47" s="232"/>
       <c r="H47" s="126"/>
       <c r="K47" s="38" t="s">
         <v>96</v>
@@ -15813,35 +15809,81 @@
       <c r="B48" s="57" t="s">
         <v>99</v>
       </c>
-      <c r="C48" s="322" t="s">
+      <c r="C48" s="235" t="s">
         <v>208</v>
       </c>
-      <c r="D48" s="322"/>
-      <c r="E48" s="322"/>
-      <c r="F48" s="321" t="s">
+      <c r="D48" s="235"/>
+      <c r="E48" s="235"/>
+      <c r="F48" s="233" t="s">
         <v>91</v>
       </c>
-      <c r="G48" s="275"/>
+      <c r="G48" s="234"/>
       <c r="H48" s="160" t="s">
         <v>212</v>
       </c>
       <c r="I48" s="58"/>
       <c r="J48" s="59"/>
-      <c r="K48" s="318"/>
-      <c r="L48" s="319"/>
-      <c r="M48" s="319"/>
-      <c r="N48" s="319"/>
-      <c r="O48" s="319"/>
-      <c r="P48" s="320"/>
+      <c r="K48" s="228"/>
+      <c r="L48" s="229"/>
+      <c r="M48" s="229"/>
+      <c r="N48" s="229"/>
+      <c r="O48" s="229"/>
+      <c r="P48" s="230"/>
     </row>
   </sheetData>
   <mergeCells count="74">
-    <mergeCell ref="D25:F25"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="D19:D20"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="K44:L44"/>
+    <mergeCell ref="N44:P44"/>
+    <mergeCell ref="L31:P31"/>
+    <mergeCell ref="L30:O30"/>
+    <mergeCell ref="L29:P29"/>
+    <mergeCell ref="B32:B33"/>
+    <mergeCell ref="L4:M4"/>
+    <mergeCell ref="L5:M5"/>
+    <mergeCell ref="L6:M6"/>
+    <mergeCell ref="L7:M7"/>
+    <mergeCell ref="C8:I8"/>
+    <mergeCell ref="L8:P8"/>
+    <mergeCell ref="C9:I10"/>
+    <mergeCell ref="C30:F31"/>
+    <mergeCell ref="N6:P7"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="L9:O10"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="M13:N13"/>
+    <mergeCell ref="M14:N14"/>
+    <mergeCell ref="L11:P12"/>
+    <mergeCell ref="D16:F16"/>
+    <mergeCell ref="A2:P2"/>
+    <mergeCell ref="N3:P3"/>
+    <mergeCell ref="C4:K4"/>
+    <mergeCell ref="C5:K5"/>
+    <mergeCell ref="C6:K6"/>
+    <mergeCell ref="C7:K7"/>
+    <mergeCell ref="N4:P5"/>
+    <mergeCell ref="K45:P45"/>
+    <mergeCell ref="C46:E46"/>
+    <mergeCell ref="K46:P46"/>
+    <mergeCell ref="H16:I16"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="C45:E45"/>
+    <mergeCell ref="F44:G44"/>
+    <mergeCell ref="F45:G45"/>
+    <mergeCell ref="C21:H21"/>
+    <mergeCell ref="C22:H22"/>
+    <mergeCell ref="O24:P24"/>
+    <mergeCell ref="O23:P23"/>
+    <mergeCell ref="L23:N23"/>
+    <mergeCell ref="L24:N24"/>
+    <mergeCell ref="C29:G29"/>
+    <mergeCell ref="H29:I29"/>
+    <mergeCell ref="K48:P48"/>
+    <mergeCell ref="F46:G46"/>
+    <mergeCell ref="F47:G47"/>
+    <mergeCell ref="F48:G48"/>
+    <mergeCell ref="C47:E47"/>
+    <mergeCell ref="C48:E48"/>
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="C44:E44"/>
     <mergeCell ref="C43:E43"/>
@@ -15858,58 +15900,12 @@
     <mergeCell ref="D27:D28"/>
     <mergeCell ref="E27:E28"/>
     <mergeCell ref="F27:F28"/>
-    <mergeCell ref="K48:P48"/>
-    <mergeCell ref="F46:G46"/>
-    <mergeCell ref="F47:G47"/>
-    <mergeCell ref="F48:G48"/>
-    <mergeCell ref="C47:E47"/>
-    <mergeCell ref="C48:E48"/>
-    <mergeCell ref="K45:P45"/>
-    <mergeCell ref="C46:E46"/>
-    <mergeCell ref="K46:P46"/>
-    <mergeCell ref="H16:I16"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="C45:E45"/>
-    <mergeCell ref="F44:G44"/>
-    <mergeCell ref="F45:G45"/>
-    <mergeCell ref="C21:H21"/>
-    <mergeCell ref="C22:H22"/>
-    <mergeCell ref="O24:P24"/>
-    <mergeCell ref="O23:P23"/>
-    <mergeCell ref="L23:N23"/>
-    <mergeCell ref="L24:N24"/>
-    <mergeCell ref="C29:G29"/>
-    <mergeCell ref="H29:I29"/>
-    <mergeCell ref="L11:P12"/>
-    <mergeCell ref="D16:F16"/>
-    <mergeCell ref="A2:P2"/>
-    <mergeCell ref="N3:P3"/>
-    <mergeCell ref="C4:K4"/>
-    <mergeCell ref="C5:K5"/>
-    <mergeCell ref="C6:K6"/>
-    <mergeCell ref="C7:K7"/>
-    <mergeCell ref="N4:P5"/>
-    <mergeCell ref="B32:B33"/>
-    <mergeCell ref="L4:M4"/>
-    <mergeCell ref="L5:M5"/>
-    <mergeCell ref="L6:M6"/>
-    <mergeCell ref="L7:M7"/>
-    <mergeCell ref="C8:I8"/>
-    <mergeCell ref="L8:P8"/>
-    <mergeCell ref="C9:I10"/>
-    <mergeCell ref="C30:F31"/>
-    <mergeCell ref="N6:P7"/>
-    <mergeCell ref="D15:F15"/>
-    <mergeCell ref="L9:O10"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="M16:N16"/>
-    <mergeCell ref="M13:N13"/>
-    <mergeCell ref="M14:N14"/>
-    <mergeCell ref="K44:L44"/>
-    <mergeCell ref="N44:P44"/>
-    <mergeCell ref="L31:P31"/>
-    <mergeCell ref="L30:O30"/>
-    <mergeCell ref="L29:P29"/>
+    <mergeCell ref="D25:F25"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="D19:D20"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="E23:F23"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.47244094488188981" right="0.23622047244094491" top="0.59055118110236227" bottom="0.70866141732283472" header="0.51181102362204722" footer="0.51181102362204722"/>
@@ -15939,43 +15935,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="39" customHeight="1">
-      <c r="A1" s="199" t="s">
+      <c r="A1" s="201" t="s">
         <v>100</v>
       </c>
-      <c r="B1" s="199"/>
-      <c r="C1" s="199"/>
-      <c r="D1" s="199"/>
-      <c r="E1" s="199"/>
-      <c r="F1" s="199"/>
-      <c r="G1" s="199"/>
-      <c r="H1" s="199"/>
-      <c r="I1" s="199"/>
-      <c r="J1" s="199"/>
-      <c r="K1" s="199"/>
-      <c r="L1" s="199"/>
-      <c r="M1" s="199"/>
-      <c r="N1" s="199"/>
-      <c r="O1" s="199"/>
-      <c r="P1" s="199"/>
-      <c r="Q1" s="199"/>
-      <c r="R1" s="199"/>
-      <c r="S1" s="199"/>
-      <c r="T1" s="199"/>
-      <c r="U1" s="199"/>
-      <c r="V1" s="199"/>
-      <c r="W1" s="199"/>
-      <c r="X1" s="199"/>
+      <c r="B1" s="201"/>
+      <c r="C1" s="201"/>
+      <c r="D1" s="201"/>
+      <c r="E1" s="201"/>
+      <c r="F1" s="201"/>
+      <c r="G1" s="201"/>
+      <c r="H1" s="201"/>
+      <c r="I1" s="201"/>
+      <c r="J1" s="201"/>
+      <c r="K1" s="201"/>
+      <c r="L1" s="201"/>
+      <c r="M1" s="201"/>
+      <c r="N1" s="201"/>
+      <c r="O1" s="201"/>
+      <c r="P1" s="201"/>
+      <c r="Q1" s="201"/>
+      <c r="R1" s="201"/>
+      <c r="S1" s="201"/>
+      <c r="T1" s="201"/>
+      <c r="U1" s="201"/>
+      <c r="V1" s="201"/>
+      <c r="W1" s="201"/>
+      <c r="X1" s="201"/>
     </row>
     <row r="2" spans="1:25" ht="14.25" customHeight="1">
-      <c r="R2" s="189" t="s">
-        <v>231</v>
-      </c>
-      <c r="S2" s="189"/>
-      <c r="T2" s="189"/>
-      <c r="U2" s="189"/>
-      <c r="V2" s="189"/>
-      <c r="W2" s="189"/>
-      <c r="X2" s="189"/>
+      <c r="R2" s="339" t="s">
+        <v>230</v>
+      </c>
+      <c r="S2" s="339"/>
+      <c r="T2" s="339"/>
+      <c r="U2" s="339"/>
+      <c r="V2" s="339"/>
+      <c r="W2" s="339"/>
+      <c r="X2" s="339"/>
     </row>
     <row r="3" spans="1:25" ht="18" customHeight="1">
       <c r="A3" s="62"/>
@@ -15999,15 +15995,15 @@
       </c>
       <c r="P3" s="65"/>
       <c r="Q3" s="54"/>
-      <c r="R3" s="203" t="s">
+      <c r="R3" s="343" t="s">
         <v>169</v>
       </c>
-      <c r="S3" s="204"/>
-      <c r="T3" s="204"/>
-      <c r="U3" s="204"/>
-      <c r="V3" s="204"/>
-      <c r="W3" s="204"/>
-      <c r="X3" s="205"/>
+      <c r="S3" s="344"/>
+      <c r="T3" s="344"/>
+      <c r="U3" s="344"/>
+      <c r="V3" s="344"/>
+      <c r="W3" s="344"/>
+      <c r="X3" s="345"/>
     </row>
     <row r="4" spans="1:25" ht="12.75" customHeight="1">
       <c r="A4" s="66"/>
@@ -16020,13 +16016,13 @@
       </c>
       <c r="P4" s="69"/>
       <c r="Q4"/>
-      <c r="R4" s="206"/>
-      <c r="S4" s="207"/>
-      <c r="T4" s="207"/>
-      <c r="U4" s="207"/>
-      <c r="V4" s="207"/>
-      <c r="W4" s="207"/>
-      <c r="X4" s="208"/>
+      <c r="R4" s="346"/>
+      <c r="S4" s="347"/>
+      <c r="T4" s="347"/>
+      <c r="U4" s="347"/>
+      <c r="V4" s="347"/>
+      <c r="W4" s="347"/>
+      <c r="X4" s="348"/>
     </row>
     <row r="5" spans="1:25" ht="13.5" customHeight="1">
       <c r="A5" s="66"/>
@@ -16038,15 +16034,15 @@
       </c>
       <c r="P5" s="70"/>
       <c r="Q5" s="16"/>
-      <c r="R5" s="209" t="s">
+      <c r="R5" s="349" t="s">
         <v>170</v>
       </c>
-      <c r="S5" s="210"/>
-      <c r="T5" s="210"/>
-      <c r="U5" s="210"/>
-      <c r="V5" s="210"/>
-      <c r="W5" s="210"/>
-      <c r="X5" s="211"/>
+      <c r="S5" s="350"/>
+      <c r="T5" s="350"/>
+      <c r="U5" s="350"/>
+      <c r="V5" s="350"/>
+      <c r="W5" s="350"/>
+      <c r="X5" s="351"/>
     </row>
     <row r="6" spans="1:25" ht="12.75" customHeight="1">
       <c r="A6" s="71"/>
@@ -16070,13 +16066,13 @@
       </c>
       <c r="P6" s="74"/>
       <c r="Q6" s="60"/>
-      <c r="R6" s="212"/>
-      <c r="S6" s="213"/>
-      <c r="T6" s="213"/>
-      <c r="U6" s="213"/>
-      <c r="V6" s="213"/>
-      <c r="W6" s="213"/>
-      <c r="X6" s="214"/>
+      <c r="R6" s="352"/>
+      <c r="S6" s="353"/>
+      <c r="T6" s="353"/>
+      <c r="U6" s="353"/>
+      <c r="V6" s="353"/>
+      <c r="W6" s="353"/>
+      <c r="X6" s="354"/>
     </row>
     <row r="7" spans="1:25" s="78" customFormat="1" ht="5.25" customHeight="1">
       <c r="A7" s="75"/>
@@ -16285,11 +16281,9 @@
       <c r="T10" s="111" t="s">
         <v>163</v>
       </c>
-      <c r="U10" s="200" t="s">
-        <v>222</v>
-      </c>
-      <c r="V10" s="201"/>
-      <c r="W10" s="202"/>
+      <c r="U10" s="336"/>
+      <c r="V10" s="337"/>
+      <c r="W10" s="338"/>
       <c r="X10" s="112"/>
     </row>
     <row r="11" spans="1:25" ht="18.899999999999999" customHeight="1">
@@ -16313,9 +16307,9 @@
       <c r="R11" s="164"/>
       <c r="S11" s="164"/>
       <c r="T11" s="167"/>
-      <c r="U11" s="196"/>
-      <c r="V11" s="197"/>
-      <c r="W11" s="198"/>
+      <c r="U11" s="330"/>
+      <c r="V11" s="331"/>
+      <c r="W11" s="332"/>
       <c r="X11" s="185"/>
     </row>
     <row r="12" spans="1:25" ht="18.899999999999999" customHeight="1">
@@ -16339,9 +16333,9 @@
       <c r="R12" s="171"/>
       <c r="S12" s="171"/>
       <c r="T12" s="172"/>
-      <c r="U12" s="190"/>
-      <c r="V12" s="191"/>
-      <c r="W12" s="192"/>
+      <c r="U12" s="333"/>
+      <c r="V12" s="334"/>
+      <c r="W12" s="335"/>
       <c r="X12" s="186"/>
     </row>
     <row r="13" spans="1:25" ht="18.899999999999999" customHeight="1">
@@ -16365,9 +16359,9 @@
       <c r="R13" s="171"/>
       <c r="S13" s="171"/>
       <c r="T13" s="172"/>
-      <c r="U13" s="190"/>
-      <c r="V13" s="191"/>
-      <c r="W13" s="192"/>
+      <c r="U13" s="333"/>
+      <c r="V13" s="334"/>
+      <c r="W13" s="335"/>
       <c r="X13" s="187"/>
     </row>
     <row r="14" spans="1:25" ht="18.899999999999999" customHeight="1">
@@ -16391,9 +16385,9 @@
       <c r="R14" s="171"/>
       <c r="S14" s="171"/>
       <c r="T14" s="172"/>
-      <c r="U14" s="190"/>
-      <c r="V14" s="191"/>
-      <c r="W14" s="192"/>
+      <c r="U14" s="333"/>
+      <c r="V14" s="334"/>
+      <c r="W14" s="335"/>
       <c r="X14" s="173"/>
     </row>
     <row r="15" spans="1:25" ht="18.899999999999999" customHeight="1">
@@ -16417,9 +16411,9 @@
       <c r="R15" s="171"/>
       <c r="S15" s="171"/>
       <c r="T15" s="172"/>
-      <c r="U15" s="190"/>
-      <c r="V15" s="191"/>
-      <c r="W15" s="192"/>
+      <c r="U15" s="333"/>
+      <c r="V15" s="334"/>
+      <c r="W15" s="335"/>
       <c r="X15" s="173"/>
     </row>
     <row r="16" spans="1:25" ht="18.899999999999999" customHeight="1">
@@ -16443,9 +16437,9 @@
       <c r="R16" s="171"/>
       <c r="S16" s="171"/>
       <c r="T16" s="172"/>
-      <c r="U16" s="190"/>
-      <c r="V16" s="191"/>
-      <c r="W16" s="192"/>
+      <c r="U16" s="333"/>
+      <c r="V16" s="334"/>
+      <c r="W16" s="335"/>
       <c r="X16" s="173"/>
     </row>
     <row r="17" spans="1:24" ht="18.899999999999999" customHeight="1">
@@ -16469,9 +16463,9 @@
       <c r="R17" s="171"/>
       <c r="S17" s="171"/>
       <c r="T17" s="172"/>
-      <c r="U17" s="196"/>
-      <c r="V17" s="197"/>
-      <c r="W17" s="198"/>
+      <c r="U17" s="330"/>
+      <c r="V17" s="331"/>
+      <c r="W17" s="332"/>
       <c r="X17" s="185"/>
     </row>
     <row r="18" spans="1:24" ht="18.899999999999999" customHeight="1">
@@ -16495,9 +16489,9 @@
       <c r="R18" s="171"/>
       <c r="S18" s="171"/>
       <c r="T18" s="172"/>
-      <c r="U18" s="196"/>
-      <c r="V18" s="197"/>
-      <c r="W18" s="198"/>
+      <c r="U18" s="330"/>
+      <c r="V18" s="331"/>
+      <c r="W18" s="332"/>
       <c r="X18" s="185"/>
     </row>
     <row r="19" spans="1:24" ht="18.899999999999999" customHeight="1">
@@ -16521,9 +16515,9 @@
       <c r="R19" s="171"/>
       <c r="S19" s="171"/>
       <c r="T19" s="172"/>
-      <c r="U19" s="190"/>
-      <c r="V19" s="191"/>
-      <c r="W19" s="192"/>
+      <c r="U19" s="333"/>
+      <c r="V19" s="334"/>
+      <c r="W19" s="335"/>
       <c r="X19" s="188"/>
     </row>
     <row r="20" spans="1:24" ht="18.899999999999999" customHeight="1">
@@ -16547,9 +16541,9 @@
       <c r="R20" s="171"/>
       <c r="S20" s="171"/>
       <c r="T20" s="172"/>
-      <c r="U20" s="196"/>
-      <c r="V20" s="197"/>
-      <c r="W20" s="198"/>
+      <c r="U20" s="330"/>
+      <c r="V20" s="331"/>
+      <c r="W20" s="332"/>
       <c r="X20" s="185"/>
     </row>
     <row r="21" spans="1:24" ht="18.899999999999999" customHeight="1">
@@ -16573,9 +16567,9 @@
       <c r="R21" s="171"/>
       <c r="S21" s="171"/>
       <c r="T21" s="172"/>
-      <c r="U21" s="196"/>
-      <c r="V21" s="197"/>
-      <c r="W21" s="198"/>
+      <c r="U21" s="330"/>
+      <c r="V21" s="331"/>
+      <c r="W21" s="332"/>
       <c r="X21" s="185"/>
     </row>
     <row r="22" spans="1:24" ht="18.899999999999999" customHeight="1">
@@ -16599,9 +16593,9 @@
       <c r="R22" s="171"/>
       <c r="S22" s="171"/>
       <c r="T22" s="172"/>
-      <c r="U22" s="190"/>
-      <c r="V22" s="191"/>
-      <c r="W22" s="192"/>
+      <c r="U22" s="333"/>
+      <c r="V22" s="334"/>
+      <c r="W22" s="335"/>
       <c r="X22" s="186"/>
     </row>
     <row r="23" spans="1:24" ht="18.899999999999999" customHeight="1">
@@ -16625,9 +16619,9 @@
       <c r="R23" s="171"/>
       <c r="S23" s="171"/>
       <c r="T23" s="172"/>
-      <c r="U23" s="196"/>
-      <c r="V23" s="197"/>
-      <c r="W23" s="198"/>
+      <c r="U23" s="330"/>
+      <c r="V23" s="331"/>
+      <c r="W23" s="332"/>
       <c r="X23" s="185"/>
     </row>
     <row r="24" spans="1:24" ht="18.899999999999999" customHeight="1">
@@ -16651,9 +16645,9 @@
       <c r="R24" s="171"/>
       <c r="S24" s="171"/>
       <c r="T24" s="172"/>
-      <c r="U24" s="196"/>
-      <c r="V24" s="197"/>
-      <c r="W24" s="198"/>
+      <c r="U24" s="330"/>
+      <c r="V24" s="331"/>
+      <c r="W24" s="332"/>
       <c r="X24" s="185"/>
     </row>
     <row r="25" spans="1:24" ht="18.899999999999999" customHeight="1">
@@ -16677,9 +16671,9 @@
       <c r="R25" s="171"/>
       <c r="S25" s="171"/>
       <c r="T25" s="172"/>
-      <c r="U25" s="196"/>
-      <c r="V25" s="197"/>
-      <c r="W25" s="198"/>
+      <c r="U25" s="330"/>
+      <c r="V25" s="331"/>
+      <c r="W25" s="332"/>
       <c r="X25" s="185"/>
     </row>
     <row r="26" spans="1:24" ht="18.899999999999999" customHeight="1">
@@ -16703,9 +16697,9 @@
       <c r="R26" s="171"/>
       <c r="S26" s="171"/>
       <c r="T26" s="172"/>
-      <c r="U26" s="190"/>
-      <c r="V26" s="191"/>
-      <c r="W26" s="192"/>
+      <c r="U26" s="333"/>
+      <c r="V26" s="334"/>
+      <c r="W26" s="335"/>
       <c r="X26" s="188"/>
     </row>
     <row r="27" spans="1:24" ht="18.899999999999999" customHeight="1">
@@ -16729,9 +16723,9 @@
       <c r="R27" s="171"/>
       <c r="S27" s="171"/>
       <c r="T27" s="172"/>
-      <c r="U27" s="196"/>
-      <c r="V27" s="197"/>
-      <c r="W27" s="198"/>
+      <c r="U27" s="330"/>
+      <c r="V27" s="331"/>
+      <c r="W27" s="332"/>
       <c r="X27" s="185"/>
     </row>
     <row r="28" spans="1:24" ht="18.899999999999999" customHeight="1">
@@ -16755,9 +16749,9 @@
       <c r="R28" s="171"/>
       <c r="S28" s="171"/>
       <c r="T28" s="172"/>
-      <c r="U28" s="190"/>
-      <c r="V28" s="191"/>
-      <c r="W28" s="192"/>
+      <c r="U28" s="333"/>
+      <c r="V28" s="334"/>
+      <c r="W28" s="335"/>
       <c r="X28" s="186"/>
     </row>
     <row r="29" spans="1:24" ht="18.899999999999999" customHeight="1">
@@ -16781,9 +16775,9 @@
       <c r="R29" s="171"/>
       <c r="S29" s="171"/>
       <c r="T29" s="172"/>
-      <c r="U29" s="196"/>
-      <c r="V29" s="197"/>
-      <c r="W29" s="198"/>
+      <c r="U29" s="330"/>
+      <c r="V29" s="331"/>
+      <c r="W29" s="332"/>
       <c r="X29" s="185"/>
     </row>
     <row r="30" spans="1:24" ht="18.899999999999999" customHeight="1">
@@ -16807,9 +16801,9 @@
       <c r="R30" s="171"/>
       <c r="S30" s="171"/>
       <c r="T30" s="172"/>
-      <c r="U30" s="196"/>
-      <c r="V30" s="197"/>
-      <c r="W30" s="198"/>
+      <c r="U30" s="330"/>
+      <c r="V30" s="331"/>
+      <c r="W30" s="332"/>
       <c r="X30" s="185"/>
     </row>
     <row r="31" spans="1:24" ht="18.899999999999999" customHeight="1">
@@ -16833,9 +16827,9 @@
       <c r="R31" s="171"/>
       <c r="S31" s="171"/>
       <c r="T31" s="172"/>
-      <c r="U31" s="190"/>
-      <c r="V31" s="191"/>
-      <c r="W31" s="192"/>
+      <c r="U31" s="333"/>
+      <c r="V31" s="334"/>
+      <c r="W31" s="335"/>
       <c r="X31" s="186"/>
     </row>
     <row r="32" spans="1:24" ht="18.899999999999999" customHeight="1">
@@ -16859,9 +16853,9 @@
       <c r="R32" s="171"/>
       <c r="S32" s="171"/>
       <c r="T32" s="172"/>
-      <c r="U32" s="196"/>
-      <c r="V32" s="197"/>
-      <c r="W32" s="198"/>
+      <c r="U32" s="330"/>
+      <c r="V32" s="331"/>
+      <c r="W32" s="332"/>
       <c r="X32" s="185"/>
     </row>
     <row r="33" spans="1:24" ht="18.899999999999999" customHeight="1">
@@ -16885,9 +16879,9 @@
       <c r="R33" s="171"/>
       <c r="S33" s="171"/>
       <c r="T33" s="172"/>
-      <c r="U33" s="196"/>
-      <c r="V33" s="197"/>
-      <c r="W33" s="198"/>
+      <c r="U33" s="330"/>
+      <c r="V33" s="331"/>
+      <c r="W33" s="332"/>
       <c r="X33" s="185"/>
     </row>
     <row r="34" spans="1:24" ht="18.899999999999999" customHeight="1">
@@ -16911,41 +16905,55 @@
       <c r="R34" s="171"/>
       <c r="S34" s="171"/>
       <c r="T34" s="172"/>
-      <c r="U34" s="190"/>
-      <c r="V34" s="191"/>
-      <c r="W34" s="192"/>
+      <c r="U34" s="333"/>
+      <c r="V34" s="334"/>
+      <c r="W34" s="335"/>
       <c r="X34" s="186"/>
     </row>
     <row r="35" spans="1:24" ht="18.899999999999999" customHeight="1">
-      <c r="A35" s="193" t="s">
+      <c r="A35" s="340" t="s">
         <v>199</v>
       </c>
-      <c r="B35" s="194"/>
-      <c r="C35" s="194"/>
-      <c r="D35" s="194"/>
-      <c r="E35" s="194"/>
-      <c r="F35" s="194"/>
-      <c r="G35" s="194"/>
-      <c r="H35" s="194"/>
-      <c r="I35" s="194"/>
-      <c r="J35" s="194"/>
-      <c r="K35" s="194"/>
-      <c r="L35" s="194"/>
-      <c r="M35" s="194"/>
-      <c r="N35" s="194"/>
-      <c r="O35" s="194"/>
-      <c r="P35" s="194"/>
-      <c r="Q35" s="194"/>
-      <c r="R35" s="194"/>
-      <c r="S35" s="194"/>
-      <c r="T35" s="194"/>
-      <c r="U35" s="194"/>
-      <c r="V35" s="194"/>
-      <c r="W35" s="194"/>
-      <c r="X35" s="195"/>
+      <c r="B35" s="341"/>
+      <c r="C35" s="341"/>
+      <c r="D35" s="341"/>
+      <c r="E35" s="341"/>
+      <c r="F35" s="341"/>
+      <c r="G35" s="341"/>
+      <c r="H35" s="341"/>
+      <c r="I35" s="341"/>
+      <c r="J35" s="341"/>
+      <c r="K35" s="341"/>
+      <c r="L35" s="341"/>
+      <c r="M35" s="341"/>
+      <c r="N35" s="341"/>
+      <c r="O35" s="341"/>
+      <c r="P35" s="341"/>
+      <c r="Q35" s="341"/>
+      <c r="R35" s="341"/>
+      <c r="S35" s="341"/>
+      <c r="T35" s="341"/>
+      <c r="U35" s="341"/>
+      <c r="V35" s="341"/>
+      <c r="W35" s="341"/>
+      <c r="X35" s="342"/>
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="R2:X2"/>
+    <mergeCell ref="U34:W34"/>
+    <mergeCell ref="A35:X35"/>
+    <mergeCell ref="U28:W28"/>
+    <mergeCell ref="U29:W29"/>
+    <mergeCell ref="U30:W30"/>
+    <mergeCell ref="U31:W31"/>
+    <mergeCell ref="U23:W23"/>
+    <mergeCell ref="R3:X4"/>
+    <mergeCell ref="R5:X6"/>
+    <mergeCell ref="U14:W14"/>
+    <mergeCell ref="U15:W15"/>
+    <mergeCell ref="U11:W11"/>
+    <mergeCell ref="U12:W12"/>
     <mergeCell ref="A1:X1"/>
     <mergeCell ref="U33:W33"/>
     <mergeCell ref="U16:W16"/>
@@ -16962,20 +16970,6 @@
     <mergeCell ref="U20:W20"/>
     <mergeCell ref="U21:W21"/>
     <mergeCell ref="U22:W22"/>
-    <mergeCell ref="R2:X2"/>
-    <mergeCell ref="U34:W34"/>
-    <mergeCell ref="A35:X35"/>
-    <mergeCell ref="U28:W28"/>
-    <mergeCell ref="U29:W29"/>
-    <mergeCell ref="U30:W30"/>
-    <mergeCell ref="U31:W31"/>
-    <mergeCell ref="U23:W23"/>
-    <mergeCell ref="R3:X4"/>
-    <mergeCell ref="R5:X6"/>
-    <mergeCell ref="U14:W14"/>
-    <mergeCell ref="U15:W15"/>
-    <mergeCell ref="U11:W11"/>
-    <mergeCell ref="U12:W12"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.47244094488188981" right="0.31496062992125984" top="0.55118110236220474" bottom="0.74803149606299213" header="0.51181102362204722" footer="0.51181102362204722"/>

</xml_diff>